<commit_message>
feat(interface) : Implémentation de l'interface utilisateur, avec toutes les données du parking affichée (pour l'instant ce sont de fausses donées)
</commit_message>
<xml_diff>
--- a/fichiers/P_parking-jdt-HugoSchweizer.xlsx
+++ b/fichiers/P_parking-jdt-HugoSchweizer.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\P_parking\fichiers\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64BCBC6C-58CE-4B3B-A935-9CA33925CEF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94DDFBBF-6545-4A4E-BFE9-01C2CBE73FAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="39">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -152,6 +152,12 @@
   </si>
   <si>
     <t>Planification finie</t>
+  </si>
+  <si>
+    <t>Initialisation C# terminée (Imaginer et créer l'interface utilisateur pour pouvoir y afficher les données dès qu'elles seront utilisables.)</t>
+  </si>
+  <si>
+    <t>Interface utilisateur finie (Avec de fausses données, il faut simplement les remplacer)</t>
   </si>
 </sst>
 </file>
@@ -1162,7 +1168,7 @@
                   <c:v>60</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>60</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -2092,16 +2098,16 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>0.30769230769230771</c:v>
+                  <c:v>0.23529411764705882</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>0.23529411764705882</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.69230769230769229</c:v>
+                  <c:v>0.52941176470588236</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -4339,7 +4345,7 @@
       <c r="B3" s="86"/>
       <c r="C3" s="67" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>3 heures 45 minutes</v>
+        <v>4 heures 45 minutes</v>
       </c>
       <c r="D3" s="17"/>
       <c r="E3" s="3"/>
@@ -4358,11 +4364,11 @@
       </c>
       <c r="D4" s="17">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>105</v>
+        <v>165</v>
       </c>
       <c r="E4" s="24">
         <f>SUM(C4:D4)</f>
-        <v>225</v>
+        <v>285</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -4407,7 +4413,9 @@
       <c r="C7" s="27">
         <v>1</v>
       </c>
-      <c r="D7" s="28"/>
+      <c r="D7" s="28">
+        <v>0</v>
+      </c>
       <c r="E7" s="29" t="s">
         <v>14</v>
       </c>
@@ -4427,7 +4435,9 @@
       <c r="C8" s="31">
         <v>1</v>
       </c>
-      <c r="D8" s="32"/>
+      <c r="D8" s="32">
+        <v>0</v>
+      </c>
       <c r="E8" s="33" t="s">
         <v>17</v>
       </c>
@@ -4559,16 +4569,22 @@
         <v>20</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:15" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A13" s="63" t="str">
         <f>IF(ISBLANK(B13),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B13))</f>
         <v/>
       </c>
       <c r="B13" s="34"/>
       <c r="C13" s="35"/>
-      <c r="D13" s="36"/>
-      <c r="E13" s="37"/>
-      <c r="F13" s="23"/>
+      <c r="D13" s="36">
+        <v>30</v>
+      </c>
+      <c r="E13" s="37" t="s">
+        <v>16</v>
+      </c>
+      <c r="F13" s="23" t="s">
+        <v>37</v>
+      </c>
       <c r="G13" s="40"/>
       <c r="N13">
         <v>6</v>
@@ -4584,9 +4600,15 @@
       </c>
       <c r="B14" s="30"/>
       <c r="C14" s="31"/>
-      <c r="D14" s="32"/>
-      <c r="E14" s="33"/>
-      <c r="F14" s="23"/>
+      <c r="D14" s="32">
+        <v>30</v>
+      </c>
+      <c r="E14" s="33" t="s">
+        <v>16</v>
+      </c>
+      <c r="F14" s="23" t="s">
+        <v>38</v>
+      </c>
       <c r="G14" s="39"/>
       <c r="N14">
         <v>7</v>
@@ -10983,7 +11005,7 @@
       </c>
       <c r="G6" s="72">
         <f>SUM(A6:B6)/$C$11</f>
-        <v>0.30769230769230771</v>
+        <v>0.23529411764705882</v>
       </c>
       <c r="L6" s="51" t="str">
         <f>'Journal de travail'!M8</f>
@@ -11004,11 +11026,11 @@
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$D$7:$D$532)</f>
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="C7">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="E7" s="73" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11016,11 +11038,11 @@
       </c>
       <c r="F7" s="74" t="str">
         <f t="shared" ref="F7:F11" si="1">QUOTIENT(SUM(A7:B7),60)&amp;" h "&amp;TEXT(MOD(SUM(A7:B7),60), "00")&amp;" min"</f>
-        <v>0 h 00 min</v>
+        <v>1 h 00 min</v>
       </c>
       <c r="G7" s="75">
         <f t="shared" ref="G7:G9" si="2">SUM(A7:B7)/$C$11</f>
-        <v>0</v>
+        <v>0.23529411764705882</v>
       </c>
       <c r="L7" s="53" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11094,7 +11116,7 @@
       </c>
       <c r="G9" s="75">
         <f t="shared" si="2"/>
-        <v>0.69230769230769229</v>
+        <v>0.52941176470588236</v>
       </c>
       <c r="L9" s="55" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11150,22 +11172,22 @@
       </c>
       <c r="B11">
         <f>SUM(B6:B10)</f>
-        <v>75</v>
+        <v>135</v>
       </c>
       <c r="C11">
         <f>SUM(A11:B11)</f>
-        <v>195</v>
+        <v>255</v>
       </c>
       <c r="E11" s="81" t="s">
         <v>29</v>
       </c>
       <c r="F11" s="71" t="str">
         <f t="shared" si="1"/>
-        <v>3 h 15 min</v>
+        <v>4 h 15 min</v>
       </c>
       <c r="G11" s="82">
         <f>C11/C12</f>
-        <v>3.6931818181818184E-2</v>
+        <v>4.8295454545454544E-2</v>
       </c>
       <c r="L11" s="56" t="s">
         <v>29</v>

</xml_diff>

<commit_message>
feat(classes) : Création et intialisation de toutes les classes nécessaire ainsi que leurs attributs respectifs et leurs concepteur
</commit_message>
<xml_diff>
--- a/fichiers/P_parking-jdt-HugoSchweizer.xlsx
+++ b/fichiers/P_parking-jdt-HugoSchweizer.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\P_parking\fichiers\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94DDFBBF-6545-4A4E-BFE9-01C2CBE73FAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6BBB9D41-D499-4D45-A238-135EE8B35E1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
+    <workbookView xWindow="2640" yWindow="2640" windowWidth="21600" windowHeight="11295" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal de travail" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="40">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -158,6 +158,9 @@
   </si>
   <si>
     <t>Interface utilisateur finie (Avec de fausses données, il faut simplement les remplacer)</t>
+  </si>
+  <si>
+    <t>J'ai créé et initailisé toutes les classes nécessaires (tous leurs attributs, et leur concepteur)</t>
   </si>
 </sst>
 </file>
@@ -1168,7 +1171,7 @@
                   <c:v>60</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>60</c:v>
+                  <c:v>150</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -2098,16 +2101,16 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>0.23529411764705882</c:v>
+                  <c:v>0.17391304347826086</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.23529411764705882</c:v>
+                  <c:v>0.43478260869565216</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.52941176470588236</c:v>
+                  <c:v>0.39130434782608697</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -4345,7 +4348,7 @@
       <c r="B3" s="86"/>
       <c r="C3" s="67" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>4 heures 45 minutes</v>
+        <v>6 heures 15 minutes</v>
       </c>
       <c r="D3" s="17"/>
       <c r="E3" s="3"/>
@@ -4360,15 +4363,15 @@
       <c r="B4" s="5"/>
       <c r="C4" s="17">
         <f>SUBTOTAL(9,$C$7:$C$531)*60</f>
-        <v>120</v>
+        <v>180</v>
       </c>
       <c r="D4" s="17">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>165</v>
+        <v>195</v>
       </c>
       <c r="E4" s="24">
         <f>SUM(C4:D4)</f>
-        <v>285</v>
+        <v>375</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -4623,10 +4626,18 @@
         <v/>
       </c>
       <c r="B15" s="34"/>
-      <c r="C15" s="35"/>
-      <c r="D15" s="36"/>
-      <c r="E15" s="37"/>
-      <c r="F15" s="23"/>
+      <c r="C15" s="35">
+        <v>1</v>
+      </c>
+      <c r="D15" s="36">
+        <v>30</v>
+      </c>
+      <c r="E15" s="37" t="s">
+        <v>16</v>
+      </c>
+      <c r="F15" s="23" t="s">
+        <v>39</v>
+      </c>
       <c r="G15" s="40"/>
       <c r="N15">
         <v>8</v>
@@ -11005,7 +11016,7 @@
       </c>
       <c r="G6" s="72">
         <f>SUM(A6:B6)/$C$11</f>
-        <v>0.23529411764705882</v>
+        <v>0.17391304347826086</v>
       </c>
       <c r="L6" s="51" t="str">
         <f>'Journal de travail'!M8</f>
@@ -11022,15 +11033,15 @@
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$C$7:$C$532)*60</f>
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$D$7:$D$532)</f>
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="C7">
         <f t="shared" si="0"/>
-        <v>60</v>
+        <v>150</v>
       </c>
       <c r="E7" s="73" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11038,11 +11049,11 @@
       </c>
       <c r="F7" s="74" t="str">
         <f t="shared" ref="F7:F11" si="1">QUOTIENT(SUM(A7:B7),60)&amp;" h "&amp;TEXT(MOD(SUM(A7:B7),60), "00")&amp;" min"</f>
-        <v>1 h 00 min</v>
+        <v>2 h 30 min</v>
       </c>
       <c r="G7" s="75">
         <f t="shared" ref="G7:G9" si="2">SUM(A7:B7)/$C$11</f>
-        <v>0.23529411764705882</v>
+        <v>0.43478260869565216</v>
       </c>
       <c r="L7" s="53" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11116,7 +11127,7 @@
       </c>
       <c r="G9" s="75">
         <f t="shared" si="2"/>
-        <v>0.52941176470588236</v>
+        <v>0.39130434782608697</v>
       </c>
       <c r="L9" s="55" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11168,26 +11179,26 @@
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11">
         <f>SUM(A6:A10)</f>
-        <v>120</v>
+        <v>180</v>
       </c>
       <c r="B11">
         <f>SUM(B6:B10)</f>
-        <v>135</v>
+        <v>165</v>
       </c>
       <c r="C11">
         <f>SUM(A11:B11)</f>
-        <v>255</v>
+        <v>345</v>
       </c>
       <c r="E11" s="81" t="s">
         <v>29</v>
       </c>
       <c r="F11" s="71" t="str">
         <f t="shared" si="1"/>
-        <v>4 h 15 min</v>
+        <v>5 h 45 min</v>
       </c>
       <c r="G11" s="82">
         <f>C11/C12</f>
-        <v>4.8295454545454544E-2</v>
+        <v>6.5340909090909088E-2</v>
       </c>
       <c r="L11" s="56" t="s">
         <v>29</v>
@@ -11226,12 +11237,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="4356f79f-5386-4bda-9d92-82d8bd7b074e" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3eb094ff-ec8d-44d8-be06-94ad3ec8832a">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -11436,20 +11449,21 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="4356f79f-5386-4bda-9d92-82d8bd7b074e" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3eb094ff-ec8d-44d8-be06-94ad3ec8832a">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="4356f79f-5386-4bda-9d92-82d8bd7b074e"/>
+    <ds:schemaRef ds:uri="3eb094ff-ec8d-44d8-be06-94ad3ec8832a"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -11474,12 +11488,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="4356f79f-5386-4bda-9d92-82d8bd7b074e"/>
-    <ds:schemaRef ds:uri="3eb094ff-ec8d-44d8-be06-94ad3ec8832a"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
feat(Entrer voiture) : on peut désormais ajouter une voiture dans le parking et l'interface se mets à jours avec le tôt de remplissage, les places occupées et les places libres, la vérification des plaques pas encore faite
</commit_message>
<xml_diff>
--- a/fichiers/P_parking-jdt-HugoSchweizer.xlsx
+++ b/fichiers/P_parking-jdt-HugoSchweizer.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\P_parking\fichiers\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6BBB9D41-D499-4D45-A238-135EE8B35E1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D5D55F6-9757-4B4F-A7BB-39CC80A4B596}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2640" yWindow="2640" windowWidth="21600" windowHeight="11295" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal de travail" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="42">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -161,6 +161,12 @@
   </si>
   <si>
     <t>J'ai créé et initailisé toutes les classes nécessaires (tous leurs attributs, et leur concepteur)</t>
+  </si>
+  <si>
+    <t>en cours de I106, pendant le temps libre</t>
+  </si>
+  <si>
+    <t>J'ai ajouté le faite de pouvoir entrer un vehicule (plus qu'as verifier si la plaque est bonne)</t>
   </si>
 </sst>
 </file>
@@ -1171,7 +1177,7 @@
                   <c:v>60</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>150</c:v>
+                  <c:v>180</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -2101,16 +2107,16 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>0.17391304347826086</c:v>
+                  <c:v>0.16</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.43478260869565216</c:v>
+                  <c:v>0.48</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.39130434782608697</c:v>
+                  <c:v>0.36</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -4348,7 +4354,7 @@
       <c r="B3" s="86"/>
       <c r="C3" s="67" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>6 heures 15 minutes</v>
+        <v>6 heures 45 minutes</v>
       </c>
       <c r="D3" s="17"/>
       <c r="E3" s="3"/>
@@ -4367,11 +4373,11 @@
       </c>
       <c r="D4" s="17">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>195</v>
+        <v>225</v>
       </c>
       <c r="E4" s="24">
         <f>SUM(C4:D4)</f>
-        <v>375</v>
+        <v>405</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -4653,10 +4659,18 @@
       </c>
       <c r="B16" s="30"/>
       <c r="C16" s="31"/>
-      <c r="D16" s="32"/>
-      <c r="E16" s="33"/>
-      <c r="F16" s="23"/>
-      <c r="G16" s="39"/>
+      <c r="D16" s="32">
+        <v>30</v>
+      </c>
+      <c r="E16" s="33" t="s">
+        <v>16</v>
+      </c>
+      <c r="F16" s="23" t="s">
+        <v>41</v>
+      </c>
+      <c r="G16" s="39" t="s">
+        <v>40</v>
+      </c>
       <c r="O16">
         <v>40</v>
       </c>
@@ -11016,7 +11030,7 @@
       </c>
       <c r="G6" s="72">
         <f>SUM(A6:B6)/$C$11</f>
-        <v>0.17391304347826086</v>
+        <v>0.16</v>
       </c>
       <c r="L6" s="51" t="str">
         <f>'Journal de travail'!M8</f>
@@ -11037,11 +11051,11 @@
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$D$7:$D$532)</f>
-        <v>90</v>
+        <v>120</v>
       </c>
       <c r="C7">
         <f t="shared" si="0"/>
-        <v>150</v>
+        <v>180</v>
       </c>
       <c r="E7" s="73" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11049,11 +11063,11 @@
       </c>
       <c r="F7" s="74" t="str">
         <f t="shared" ref="F7:F11" si="1">QUOTIENT(SUM(A7:B7),60)&amp;" h "&amp;TEXT(MOD(SUM(A7:B7),60), "00")&amp;" min"</f>
-        <v>2 h 30 min</v>
+        <v>3 h 00 min</v>
       </c>
       <c r="G7" s="75">
         <f t="shared" ref="G7:G9" si="2">SUM(A7:B7)/$C$11</f>
-        <v>0.43478260869565216</v>
+        <v>0.48</v>
       </c>
       <c r="L7" s="53" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11127,7 +11141,7 @@
       </c>
       <c r="G9" s="75">
         <f t="shared" si="2"/>
-        <v>0.39130434782608697</v>
+        <v>0.36</v>
       </c>
       <c r="L9" s="55" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11183,22 +11197,22 @@
       </c>
       <c r="B11">
         <f>SUM(B6:B10)</f>
-        <v>165</v>
+        <v>195</v>
       </c>
       <c r="C11">
         <f>SUM(A11:B11)</f>
-        <v>345</v>
+        <v>375</v>
       </c>
       <c r="E11" s="81" t="s">
         <v>29</v>
       </c>
       <c r="F11" s="71" t="str">
         <f t="shared" si="1"/>
-        <v>5 h 45 min</v>
+        <v>6 h 15 min</v>
       </c>
       <c r="G11" s="82">
         <f>C11/C12</f>
-        <v>6.5340909090909088E-2</v>
+        <v>7.1022727272727279E-2</v>
       </c>
       <c r="L11" s="56" t="s">
         <v>29</v>
@@ -11237,14 +11251,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="4356f79f-5386-4bda-9d92-82d8bd7b074e" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3eb094ff-ec8d-44d8-be06-94ad3ec8832a">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -11449,21 +11461,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="4356f79f-5386-4bda-9d92-82d8bd7b074e" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3eb094ff-ec8d-44d8-be06-94ad3ec8832a">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="4356f79f-5386-4bda-9d92-82d8bd7b074e"/>
-    <ds:schemaRef ds:uri="3eb094ff-ec8d-44d8-be06-94ad3ec8832a"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -11488,9 +11499,12 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="4356f79f-5386-4bda-9d92-82d8bd7b074e"/>
+    <ds:schemaRef ds:uri="3eb094ff-ec8d-44d8-be06-94ad3ec8832a"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
feat(vérification plaque) : vérification des plaque d'immatricualtion réussi et permet de renvoyer trois cas d'erreurs
</commit_message>
<xml_diff>
--- a/fichiers/P_parking-jdt-HugoSchweizer.xlsx
+++ b/fichiers/P_parking-jdt-HugoSchweizer.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\P_parking\fichiers\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D5D55F6-9757-4B4F-A7BB-39CC80A4B596}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AB4EFBF-6FFB-40D1-92C3-82B399C31979}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="43">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -167,6 +167,9 @@
   </si>
   <si>
     <t>J'ai ajouté le faite de pouvoir entrer un vehicule (plus qu'as verifier si la plaque est bonne)</t>
+  </si>
+  <si>
+    <t>Vérification de la plaque d'immatriculation faite</t>
   </si>
 </sst>
 </file>
@@ -1177,7 +1180,7 @@
                   <c:v>60</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>180</c:v>
+                  <c:v>210</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -2107,16 +2110,16 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>0.16</c:v>
+                  <c:v>0.14814814814814814</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.48</c:v>
+                  <c:v>0.51851851851851849</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.36</c:v>
+                  <c:v>0.33333333333333331</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -4354,7 +4357,7 @@
       <c r="B3" s="86"/>
       <c r="C3" s="67" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>6 heures 45 minutes</v>
+        <v>7 heures 15 minutes</v>
       </c>
       <c r="D3" s="17"/>
       <c r="E3" s="3"/>
@@ -4373,11 +4376,11 @@
       </c>
       <c r="D4" s="17">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>225</v>
+        <v>255</v>
       </c>
       <c r="E4" s="24">
         <f>SUM(C4:D4)</f>
-        <v>405</v>
+        <v>435</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -4682,10 +4685,18 @@
       </c>
       <c r="B17" s="34"/>
       <c r="C17" s="35"/>
-      <c r="D17" s="36"/>
-      <c r="E17" s="37"/>
-      <c r="F17" s="23"/>
-      <c r="G17" s="40"/>
+      <c r="D17" s="36">
+        <v>30</v>
+      </c>
+      <c r="E17" s="37" t="s">
+        <v>16</v>
+      </c>
+      <c r="F17" s="23" t="s">
+        <v>42</v>
+      </c>
+      <c r="G17" s="40" t="s">
+        <v>40</v>
+      </c>
       <c r="O17">
         <v>45</v>
       </c>
@@ -11030,7 +11041,7 @@
       </c>
       <c r="G6" s="72">
         <f>SUM(A6:B6)/$C$11</f>
-        <v>0.16</v>
+        <v>0.14814814814814814</v>
       </c>
       <c r="L6" s="51" t="str">
         <f>'Journal de travail'!M8</f>
@@ -11051,11 +11062,11 @@
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$D$7:$D$532)</f>
-        <v>120</v>
+        <v>150</v>
       </c>
       <c r="C7">
         <f t="shared" si="0"/>
-        <v>180</v>
+        <v>210</v>
       </c>
       <c r="E7" s="73" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11063,11 +11074,11 @@
       </c>
       <c r="F7" s="74" t="str">
         <f t="shared" ref="F7:F11" si="1">QUOTIENT(SUM(A7:B7),60)&amp;" h "&amp;TEXT(MOD(SUM(A7:B7),60), "00")&amp;" min"</f>
-        <v>3 h 00 min</v>
+        <v>3 h 30 min</v>
       </c>
       <c r="G7" s="75">
         <f t="shared" ref="G7:G9" si="2">SUM(A7:B7)/$C$11</f>
-        <v>0.48</v>
+        <v>0.51851851851851849</v>
       </c>
       <c r="L7" s="53" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11141,7 +11152,7 @@
       </c>
       <c r="G9" s="75">
         <f t="shared" si="2"/>
-        <v>0.36</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="L9" s="55" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11197,22 +11208,22 @@
       </c>
       <c r="B11">
         <f>SUM(B6:B10)</f>
-        <v>195</v>
+        <v>225</v>
       </c>
       <c r="C11">
         <f>SUM(A11:B11)</f>
-        <v>375</v>
+        <v>405</v>
       </c>
       <c r="E11" s="81" t="s">
         <v>29</v>
       </c>
       <c r="F11" s="71" t="str">
         <f t="shared" si="1"/>
-        <v>6 h 15 min</v>
+        <v>6 h 45 min</v>
       </c>
       <c r="G11" s="82">
         <f>C11/C12</f>
-        <v>7.1022727272727279E-2</v>
+        <v>7.6704545454545456E-2</v>
       </c>
       <c r="L11" s="56" t="s">
         <v>29</v>
@@ -11251,12 +11262,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="4356f79f-5386-4bda-9d92-82d8bd7b074e" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3eb094ff-ec8d-44d8-be06-94ad3ec8832a">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -11461,20 +11474,21 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="4356f79f-5386-4bda-9d92-82d8bd7b074e" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3eb094ff-ec8d-44d8-be06-94ad3ec8832a">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="4356f79f-5386-4bda-9d92-82d8bd7b074e"/>
+    <ds:schemaRef ds:uri="3eb094ff-ec8d-44d8-be06-94ad3ec8832a"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -11499,12 +11513,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="4356f79f-5386-4bda-9d92-82d8bd7b074e"/>
-    <ds:schemaRef ds:uri="3eb094ff-ec8d-44d8-be06-94ad3ec8832a"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
feat(Exitvehicule) : L'option pour faire sortir un vehicule fonctionne totalement, avec des messages d'erreur personnalisé selon le cas
</commit_message>
<xml_diff>
--- a/fichiers/P_parking-jdt-HugoSchweizer.xlsx
+++ b/fichiers/P_parking-jdt-HugoSchweizer.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\P_parking\fichiers\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AB4EFBF-6FFB-40D1-92C3-82B399C31979}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AE1DC44-BBA7-472C-91F6-8D1C7807CBB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="45">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -170,6 +170,12 @@
   </si>
   <si>
     <t>Vérification de la plaque d'immatriculation faite</t>
+  </si>
+  <si>
+    <t>Vérification de la plaque d'immatriculation améliorée ( je me suis rendu compte qu'elle ne gérait pas tout les cas) et création du ticket faite</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sortie d'un véhicule finie, il y a différents messages d'erreurs si le véhicule n'est pas dans le parking ou si la place est déjà libre. Ça nous demande bien si on est sur de vouloir sortir la voiture et nous affiche toutes les informations qui sont en relation. </t>
   </si>
 </sst>
 </file>
@@ -1180,7 +1186,7 @@
                   <c:v>60</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>210</c:v>
+                  <c:v>360</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -2110,16 +2116,16 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>0.14814814814814814</c:v>
+                  <c:v>0.10810810810810811</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.51851851851851849</c:v>
+                  <c:v>0.64864864864864868</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.33333333333333331</c:v>
+                  <c:v>0.24324324324324326</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -4357,7 +4363,7 @@
       <c r="B3" s="86"/>
       <c r="C3" s="67" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>7 heures 15 minutes</v>
+        <v>9 heures 45 minutes</v>
       </c>
       <c r="D3" s="17"/>
       <c r="E3" s="3"/>
@@ -4372,15 +4378,15 @@
       <c r="B4" s="5"/>
       <c r="C4" s="17">
         <f>SUBTOTAL(9,$C$7:$C$531)*60</f>
-        <v>180</v>
+        <v>300</v>
       </c>
       <c r="D4" s="17">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>255</v>
+        <v>285</v>
       </c>
       <c r="E4" s="24">
         <f>SUM(C4:D4)</f>
-        <v>435</v>
+        <v>585</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -4701,31 +4707,47 @@
         <v>45</v>
       </c>
     </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:15" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A18" s="62" t="str">
         <f>IF(ISBLANK(B18),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B18))</f>
         <v/>
       </c>
       <c r="B18" s="30"/>
-      <c r="C18" s="31"/>
-      <c r="D18" s="32"/>
-      <c r="E18" s="33"/>
-      <c r="F18" s="23"/>
+      <c r="C18" s="31">
+        <v>1</v>
+      </c>
+      <c r="D18" s="32">
+        <v>0</v>
+      </c>
+      <c r="E18" s="33" t="s">
+        <v>16</v>
+      </c>
+      <c r="F18" s="23" t="s">
+        <v>43</v>
+      </c>
       <c r="G18" s="39"/>
       <c r="O18">
         <v>50</v>
       </c>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:15" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A19" s="63" t="str">
         <f>IF(ISBLANK(B19),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B19))</f>
         <v/>
       </c>
       <c r="B19" s="34"/>
-      <c r="C19" s="35"/>
-      <c r="D19" s="36"/>
-      <c r="E19" s="37"/>
-      <c r="F19" s="23"/>
+      <c r="C19" s="35">
+        <v>1</v>
+      </c>
+      <c r="D19" s="36">
+        <v>30</v>
+      </c>
+      <c r="E19" s="37" t="s">
+        <v>16</v>
+      </c>
+      <c r="F19" s="23" t="s">
+        <v>44</v>
+      </c>
       <c r="G19" s="40"/>
       <c r="O19">
         <v>55</v>
@@ -11041,7 +11063,7 @@
       </c>
       <c r="G6" s="72">
         <f>SUM(A6:B6)/$C$11</f>
-        <v>0.14814814814814814</v>
+        <v>0.10810810810810811</v>
       </c>
       <c r="L6" s="51" t="str">
         <f>'Journal de travail'!M8</f>
@@ -11058,15 +11080,15 @@
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$C$7:$C$532)*60</f>
-        <v>60</v>
+        <v>180</v>
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$D$7:$D$532)</f>
-        <v>150</v>
+        <v>180</v>
       </c>
       <c r="C7">
         <f t="shared" si="0"/>
-        <v>210</v>
+        <v>360</v>
       </c>
       <c r="E7" s="73" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11074,11 +11096,11 @@
       </c>
       <c r="F7" s="74" t="str">
         <f t="shared" ref="F7:F11" si="1">QUOTIENT(SUM(A7:B7),60)&amp;" h "&amp;TEXT(MOD(SUM(A7:B7),60), "00")&amp;" min"</f>
-        <v>3 h 30 min</v>
+        <v>6 h 00 min</v>
       </c>
       <c r="G7" s="75">
         <f t="shared" ref="G7:G9" si="2">SUM(A7:B7)/$C$11</f>
-        <v>0.51851851851851849</v>
+        <v>0.64864864864864868</v>
       </c>
       <c r="L7" s="53" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11152,7 +11174,7 @@
       </c>
       <c r="G9" s="75">
         <f t="shared" si="2"/>
-        <v>0.33333333333333331</v>
+        <v>0.24324324324324326</v>
       </c>
       <c r="L9" s="55" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11204,26 +11226,26 @@
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11">
         <f>SUM(A6:A10)</f>
-        <v>180</v>
+        <v>300</v>
       </c>
       <c r="B11">
         <f>SUM(B6:B10)</f>
-        <v>225</v>
+        <v>255</v>
       </c>
       <c r="C11">
         <f>SUM(A11:B11)</f>
-        <v>405</v>
+        <v>555</v>
       </c>
       <c r="E11" s="81" t="s">
         <v>29</v>
       </c>
       <c r="F11" s="71" t="str">
         <f t="shared" si="1"/>
-        <v>6 h 45 min</v>
+        <v>9 h 15 min</v>
       </c>
       <c r="G11" s="82">
         <f>C11/C12</f>
-        <v>7.6704545454545456E-2</v>
+        <v>0.10511363636363637</v>
       </c>
       <c r="L11" s="56" t="s">
         <v>29</v>

</xml_diff>

<commit_message>
feat(affichage parking) : Possibilité d'afficher le parking graphiquement avec le numero de chaque places et une indiqucation si elle est occupée ou non
</commit_message>
<xml_diff>
--- a/fichiers/P_parking-jdt-HugoSchweizer.xlsx
+++ b/fichiers/P_parking-jdt-HugoSchweizer.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\P_parking\fichiers\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AE1DC44-BBA7-472C-91F6-8D1C7807CBB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AC6645A-AB70-4A7E-8D43-100C4703D9F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="47">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -176,6 +176,12 @@
   </si>
   <si>
     <t xml:space="preserve">Sortie d'un véhicule finie, il y a différents messages d'erreurs si le véhicule n'est pas dans le parking ou si la place est déjà libre. Ça nous demande bien si on est sur de vouloir sortir la voiture et nous affiche toutes les informations qui sont en relation. </t>
+  </si>
+  <si>
+    <t>Affichage du parking graphiquement avec les numeros de place et une indications de si elles sont libres ou non.</t>
+  </si>
+  <si>
+    <t>Fait à moitié en cours I106, pendant le temps libre</t>
   </si>
 </sst>
 </file>
@@ -1186,7 +1192,7 @@
                   <c:v>60</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>360</c:v>
+                  <c:v>420</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -2116,16 +2122,16 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>0.10810810810810811</c:v>
+                  <c:v>9.7560975609756101E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.64864864864864868</c:v>
+                  <c:v>0.68292682926829273</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.24324324324324326</c:v>
+                  <c:v>0.21951219512195122</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -4363,7 +4369,7 @@
       <c r="B3" s="86"/>
       <c r="C3" s="67" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>9 heures 45 minutes</v>
+        <v>10 heures 45 minutes</v>
       </c>
       <c r="D3" s="17"/>
       <c r="E3" s="3"/>
@@ -4378,7 +4384,7 @@
       <c r="B4" s="5"/>
       <c r="C4" s="17">
         <f>SUBTOTAL(9,$C$7:$C$531)*60</f>
-        <v>300</v>
+        <v>360</v>
       </c>
       <c r="D4" s="17">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
@@ -4386,7 +4392,7 @@
       </c>
       <c r="E4" s="24">
         <f>SUM(C4:D4)</f>
-        <v>585</v>
+        <v>645</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -4753,17 +4759,27 @@
         <v>55</v>
       </c>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:15" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A20" s="62" t="str">
         <f>IF(ISBLANK(B20),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B20))</f>
         <v/>
       </c>
       <c r="B20" s="30"/>
-      <c r="C20" s="31"/>
-      <c r="D20" s="32"/>
-      <c r="E20" s="33"/>
-      <c r="F20" s="23"/>
-      <c r="G20" s="39"/>
+      <c r="C20" s="31">
+        <v>1</v>
+      </c>
+      <c r="D20" s="32">
+        <v>0</v>
+      </c>
+      <c r="E20" s="33" t="s">
+        <v>16</v>
+      </c>
+      <c r="F20" s="23" t="s">
+        <v>45</v>
+      </c>
+      <c r="G20" s="39" t="s">
+        <v>46</v>
+      </c>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A21" s="63" t="str">
@@ -11063,7 +11079,7 @@
       </c>
       <c r="G6" s="72">
         <f>SUM(A6:B6)/$C$11</f>
-        <v>0.10810810810810811</v>
+        <v>9.7560975609756101E-2</v>
       </c>
       <c r="L6" s="51" t="str">
         <f>'Journal de travail'!M8</f>
@@ -11080,7 +11096,7 @@
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$C$7:$C$532)*60</f>
-        <v>180</v>
+        <v>240</v>
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$D$7:$D$532)</f>
@@ -11088,7 +11104,7 @@
       </c>
       <c r="C7">
         <f t="shared" si="0"/>
-        <v>360</v>
+        <v>420</v>
       </c>
       <c r="E7" s="73" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11096,11 +11112,11 @@
       </c>
       <c r="F7" s="74" t="str">
         <f t="shared" ref="F7:F11" si="1">QUOTIENT(SUM(A7:B7),60)&amp;" h "&amp;TEXT(MOD(SUM(A7:B7),60), "00")&amp;" min"</f>
-        <v>6 h 00 min</v>
+        <v>7 h 00 min</v>
       </c>
       <c r="G7" s="75">
         <f t="shared" ref="G7:G9" si="2">SUM(A7:B7)/$C$11</f>
-        <v>0.64864864864864868</v>
+        <v>0.68292682926829273</v>
       </c>
       <c r="L7" s="53" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11174,7 +11190,7 @@
       </c>
       <c r="G9" s="75">
         <f t="shared" si="2"/>
-        <v>0.24324324324324326</v>
+        <v>0.21951219512195122</v>
       </c>
       <c r="L9" s="55" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11226,7 +11242,7 @@
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11">
         <f>SUM(A6:A10)</f>
-        <v>300</v>
+        <v>360</v>
       </c>
       <c r="B11">
         <f>SUM(B6:B10)</f>
@@ -11234,18 +11250,18 @@
       </c>
       <c r="C11">
         <f>SUM(A11:B11)</f>
-        <v>555</v>
+        <v>615</v>
       </c>
       <c r="E11" s="81" t="s">
         <v>29</v>
       </c>
       <c r="F11" s="71" t="str">
         <f t="shared" si="1"/>
-        <v>9 h 15 min</v>
+        <v>10 h 15 min</v>
       </c>
       <c r="G11" s="82">
         <f>C11/C12</f>
-        <v>0.10511363636363637</v>
+        <v>0.11647727272727272</v>
       </c>
       <c r="L11" s="56" t="s">
         <v>29</v>
@@ -11284,14 +11300,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="4356f79f-5386-4bda-9d92-82d8bd7b074e" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3eb094ff-ec8d-44d8-be06-94ad3ec8832a">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -11496,21 +11510,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="4356f79f-5386-4bda-9d92-82d8bd7b074e" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3eb094ff-ec8d-44d8-be06-94ad3ec8832a">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="4356f79f-5386-4bda-9d92-82d8bd7b074e"/>
-    <ds:schemaRef ds:uri="3eb094ff-ec8d-44d8-be06-94ad3ec8832a"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -11535,9 +11548,12 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="4356f79f-5386-4bda-9d92-82d8bd7b074e"/>
+    <ds:schemaRef ds:uri="3eb094ff-ec8d-44d8-be06-94ad3ec8832a"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
feat(SearchVehicule) : On peut désormais rechercher un vehicule et s'il est dans le parking, affiche toutes les informations le concerant et son ticket actuelle, pas les anciens ticket qui ont déjà été payé.
</commit_message>
<xml_diff>
--- a/fichiers/P_parking-jdt-HugoSchweizer.xlsx
+++ b/fichiers/P_parking-jdt-HugoSchweizer.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\P_parking\fichiers\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AC6645A-AB70-4A7E-8D43-100C4703D9F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C27165C8-F27F-411C-924F-81C58150329D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="48">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -182,6 +182,9 @@
   </si>
   <si>
     <t>Fait à moitié en cours I106, pendant le temps libre</t>
+  </si>
+  <si>
+    <t>Recherche d'un vehicule dans le parking, affiche les informations du vehicule si réussi et de son ticket actuelle ( si il était déjà venu dans le parking au paravent, cet ancien ticket ne sera pas affiché).</t>
   </si>
 </sst>
 </file>
@@ -1192,7 +1195,7 @@
                   <c:v>60</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>420</c:v>
+                  <c:v>450</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -2122,16 +2125,16 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>9.7560975609756101E-2</c:v>
+                  <c:v>9.3023255813953487E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.68292682926829273</c:v>
+                  <c:v>0.69767441860465118</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.21951219512195122</c:v>
+                  <c:v>0.20930232558139536</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -4369,7 +4372,7 @@
       <c r="B3" s="86"/>
       <c r="C3" s="67" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>10 heures 45 minutes</v>
+        <v>11 heures 15 minutes</v>
       </c>
       <c r="D3" s="17"/>
       <c r="E3" s="3"/>
@@ -4388,11 +4391,11 @@
       </c>
       <c r="D4" s="17">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>285</v>
+        <v>315</v>
       </c>
       <c r="E4" s="24">
         <f>SUM(C4:D4)</f>
-        <v>645</v>
+        <v>675</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -4781,16 +4784,22 @@
         <v>46</v>
       </c>
     </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:15" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A21" s="63" t="str">
         <f>IF(ISBLANK(B21),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B21))</f>
         <v/>
       </c>
       <c r="B21" s="34"/>
       <c r="C21" s="35"/>
-      <c r="D21" s="36"/>
-      <c r="E21" s="37"/>
-      <c r="F21" s="23"/>
+      <c r="D21" s="36">
+        <v>30</v>
+      </c>
+      <c r="E21" s="37" t="s">
+        <v>16</v>
+      </c>
+      <c r="F21" s="23" t="s">
+        <v>47</v>
+      </c>
       <c r="G21" s="40"/>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
@@ -11079,7 +11088,7 @@
       </c>
       <c r="G6" s="72">
         <f>SUM(A6:B6)/$C$11</f>
-        <v>9.7560975609756101E-2</v>
+        <v>9.3023255813953487E-2</v>
       </c>
       <c r="L6" s="51" t="str">
         <f>'Journal de travail'!M8</f>
@@ -11100,11 +11109,11 @@
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$D$7:$D$532)</f>
-        <v>180</v>
+        <v>210</v>
       </c>
       <c r="C7">
         <f t="shared" si="0"/>
-        <v>420</v>
+        <v>450</v>
       </c>
       <c r="E7" s="73" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11112,11 +11121,11 @@
       </c>
       <c r="F7" s="74" t="str">
         <f t="shared" ref="F7:F11" si="1">QUOTIENT(SUM(A7:B7),60)&amp;" h "&amp;TEXT(MOD(SUM(A7:B7),60), "00")&amp;" min"</f>
-        <v>7 h 00 min</v>
+        <v>7 h 30 min</v>
       </c>
       <c r="G7" s="75">
         <f t="shared" ref="G7:G9" si="2">SUM(A7:B7)/$C$11</f>
-        <v>0.68292682926829273</v>
+        <v>0.69767441860465118</v>
       </c>
       <c r="L7" s="53" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11190,7 +11199,7 @@
       </c>
       <c r="G9" s="75">
         <f t="shared" si="2"/>
-        <v>0.21951219512195122</v>
+        <v>0.20930232558139536</v>
       </c>
       <c r="L9" s="55" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11246,22 +11255,22 @@
       </c>
       <c r="B11">
         <f>SUM(B6:B10)</f>
-        <v>255</v>
+        <v>285</v>
       </c>
       <c r="C11">
         <f>SUM(A11:B11)</f>
-        <v>615</v>
+        <v>645</v>
       </c>
       <c r="E11" s="81" t="s">
         <v>29</v>
       </c>
       <c r="F11" s="71" t="str">
         <f t="shared" si="1"/>
-        <v>10 h 15 min</v>
+        <v>10 h 45 min</v>
       </c>
       <c r="G11" s="82">
         <f>C11/C12</f>
-        <v>0.11647727272727272</v>
+        <v>0.12215909090909091</v>
       </c>
       <c r="L11" s="56" t="s">
         <v>29</v>
@@ -11300,12 +11309,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="4356f79f-5386-4bda-9d92-82d8bd7b074e" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3eb094ff-ec8d-44d8-be06-94ad3ec8832a">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -11510,20 +11521,21 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="4356f79f-5386-4bda-9d92-82d8bd7b074e" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3eb094ff-ec8d-44d8-be06-94ad3ec8832a">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="4356f79f-5386-4bda-9d92-82d8bd7b074e"/>
+    <ds:schemaRef ds:uri="3eb094ff-ec8d-44d8-be06-94ad3ec8832a"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -11548,12 +11560,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="4356f79f-5386-4bda-9d92-82d8bd7b074e"/>
-    <ds:schemaRef ds:uri="3eb094ff-ec8d-44d8-be06-94ad3ec8832a"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
feat(CloseApp) : Ferme l'application si on met une valeur qui est endehors des options affichée sur le menu, demande une confirmation, ferme l'application si validé
</commit_message>
<xml_diff>
--- a/fichiers/P_parking-jdt-HugoSchweizer.xlsx
+++ b/fichiers/P_parking-jdt-HugoSchweizer.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\P_parking\fichiers\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C27165C8-F27F-411C-924F-81C58150329D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4179C5CC-D45A-4171-8314-F8B79AC5B5E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="49">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -185,6 +185,9 @@
   </si>
   <si>
     <t>Recherche d'un vehicule dans le parking, affiche les informations du vehicule si réussi et de son ticket actuelle ( si il était déjà venu dans le parking au paravent, cet ancien ticket ne sera pas affiché).</t>
+  </si>
+  <si>
+    <t>Fermet l'application si on met autre chose que les options affichée et qu'on dise "oui".</t>
   </si>
 </sst>
 </file>
@@ -1195,7 +1198,7 @@
                   <c:v>60</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>450</c:v>
+                  <c:v>470</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -2125,16 +2128,16 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>9.3023255813953487E-2</c:v>
+                  <c:v>9.0225563909774431E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.69767441860465118</c:v>
+                  <c:v>0.70676691729323304</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.20930232558139536</c:v>
+                  <c:v>0.20300751879699247</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -4372,7 +4375,7 @@
       <c r="B3" s="86"/>
       <c r="C3" s="67" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>11 heures 15 minutes</v>
+        <v>11 heures 35 minutes</v>
       </c>
       <c r="D3" s="17"/>
       <c r="E3" s="3"/>
@@ -4391,11 +4394,11 @@
       </c>
       <c r="D4" s="17">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>315</v>
+        <v>335</v>
       </c>
       <c r="E4" s="24">
         <f>SUM(C4:D4)</f>
-        <v>675</v>
+        <v>695</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -4809,9 +4812,15 @@
       </c>
       <c r="B22" s="30"/>
       <c r="C22" s="31"/>
-      <c r="D22" s="32"/>
-      <c r="E22" s="33"/>
-      <c r="F22" s="23"/>
+      <c r="D22" s="32">
+        <v>20</v>
+      </c>
+      <c r="E22" s="33" t="s">
+        <v>16</v>
+      </c>
+      <c r="F22" s="23" t="s">
+        <v>48</v>
+      </c>
       <c r="G22" s="39"/>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.25">
@@ -11088,7 +11097,7 @@
       </c>
       <c r="G6" s="72">
         <f>SUM(A6:B6)/$C$11</f>
-        <v>9.3023255813953487E-2</v>
+        <v>9.0225563909774431E-2</v>
       </c>
       <c r="L6" s="51" t="str">
         <f>'Journal de travail'!M8</f>
@@ -11109,11 +11118,11 @@
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$D$7:$D$532)</f>
-        <v>210</v>
+        <v>230</v>
       </c>
       <c r="C7">
         <f t="shared" si="0"/>
-        <v>450</v>
+        <v>470</v>
       </c>
       <c r="E7" s="73" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11121,11 +11130,11 @@
       </c>
       <c r="F7" s="74" t="str">
         <f t="shared" ref="F7:F11" si="1">QUOTIENT(SUM(A7:B7),60)&amp;" h "&amp;TEXT(MOD(SUM(A7:B7),60), "00")&amp;" min"</f>
-        <v>7 h 30 min</v>
+        <v>7 h 50 min</v>
       </c>
       <c r="G7" s="75">
         <f t="shared" ref="G7:G9" si="2">SUM(A7:B7)/$C$11</f>
-        <v>0.69767441860465118</v>
+        <v>0.70676691729323304</v>
       </c>
       <c r="L7" s="53" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11199,7 +11208,7 @@
       </c>
       <c r="G9" s="75">
         <f t="shared" si="2"/>
-        <v>0.20930232558139536</v>
+        <v>0.20300751879699247</v>
       </c>
       <c r="L9" s="55" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11255,22 +11264,22 @@
       </c>
       <c r="B11">
         <f>SUM(B6:B10)</f>
-        <v>285</v>
+        <v>305</v>
       </c>
       <c r="C11">
         <f>SUM(A11:B11)</f>
-        <v>645</v>
+        <v>665</v>
       </c>
       <c r="E11" s="81" t="s">
         <v>29</v>
       </c>
       <c r="F11" s="71" t="str">
         <f t="shared" si="1"/>
-        <v>10 h 45 min</v>
+        <v>11 h 05 min</v>
       </c>
       <c r="G11" s="82">
         <f>C11/C12</f>
-        <v>0.12215909090909091</v>
+        <v>0.1259469696969697</v>
       </c>
       <c r="L11" s="56" t="s">
         <v>29</v>
@@ -11309,14 +11318,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="4356f79f-5386-4bda-9d92-82d8bd7b074e" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3eb094ff-ec8d-44d8-be06-94ad3ec8832a">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -11521,21 +11528,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="4356f79f-5386-4bda-9d92-82d8bd7b074e" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3eb094ff-ec8d-44d8-be06-94ad3ec8832a">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="4356f79f-5386-4bda-9d92-82d8bd7b074e"/>
-    <ds:schemaRef ds:uri="3eb094ff-ec8d-44d8-be06-94ad3ec8832a"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -11560,9 +11566,12 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="4356f79f-5386-4bda-9d92-82d8bd7b074e"/>
+    <ds:schemaRef ds:uri="3eb094ff-ec8d-44d8-be06-94ad3ec8832a"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
refactor(ShowParking) : J'ai modifié le calcule du temps et le calcule du prix du ticket qui n'était pas du tout correcte, et j'ai aussi ajouté un prix de ticket minimum. L'affiche du ticket aussi à été modifié ainsi que les véhicules présents dans le parking quand on affiche le parking.
</commit_message>
<xml_diff>
--- a/fichiers/P_parking-jdt-HugoSchweizer.xlsx
+++ b/fichiers/P_parking-jdt-HugoSchweizer.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\P_parking\fichiers\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4179C5CC-D45A-4171-8314-F8B79AC5B5E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AB65B42-7C57-4C36-A188-02576AC76E7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="50">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -187,7 +187,10 @@
     <t>Recherche d'un vehicule dans le parking, affiche les informations du vehicule si réussi et de son ticket actuelle ( si il était déjà venu dans le parking au paravent, cet ancien ticket ne sera pas affiché).</t>
   </si>
   <si>
-    <t>Fermet l'application si on met autre chose que les options affichée et qu'on dise "oui".</t>
+    <t>Fermer l'application si on met autre chose que les options affichée et qu'on dise "oui".</t>
+  </si>
+  <si>
+    <t>J'ai modifié le calcule du temps et le calcule du prix du ticket qui n'était pas du tout correcte, et j'ai aussi ajouté un prix de ticket minimum. L'affiche du ticket aussi à été modifié ainsi que les véhicules présents dans le parking quand on affiche le parking.</t>
   </si>
 </sst>
 </file>
@@ -1198,7 +1201,7 @@
                   <c:v>60</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>470</c:v>
+                  <c:v>620</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -2128,16 +2131,16 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>9.0225563909774431E-2</c:v>
+                  <c:v>7.3619631901840496E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.70676691729323304</c:v>
+                  <c:v>0.76073619631901845</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.20300751879699247</c:v>
+                  <c:v>0.16564417177914109</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -4375,7 +4378,7 @@
       <c r="B3" s="86"/>
       <c r="C3" s="67" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>11 heures 35 minutes</v>
+        <v>14 heures 5 minutes</v>
       </c>
       <c r="D3" s="17"/>
       <c r="E3" s="3"/>
@@ -4390,15 +4393,15 @@
       <c r="B4" s="5"/>
       <c r="C4" s="17">
         <f>SUBTOTAL(9,$C$7:$C$531)*60</f>
-        <v>360</v>
+        <v>480</v>
       </c>
       <c r="D4" s="17">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>335</v>
+        <v>365</v>
       </c>
       <c r="E4" s="24">
         <f>SUM(C4:D4)</f>
-        <v>695</v>
+        <v>845</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -4600,11 +4603,13 @@
       </c>
     </row>
     <row r="13" spans="1:15" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A13" s="63" t="str">
+      <c r="A13" s="63">
         <f>IF(ISBLANK(B13),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B13))</f>
-        <v/>
-      </c>
-      <c r="B13" s="34"/>
+        <v>36</v>
+      </c>
+      <c r="B13" s="34">
+        <v>46269</v>
+      </c>
       <c r="C13" s="35"/>
       <c r="D13" s="36">
         <v>30</v>
@@ -4624,11 +4629,13 @@
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A14" s="62" t="str">
+      <c r="A14" s="62">
         <f>IF(ISBLANK(B14),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B14))</f>
-        <v/>
-      </c>
-      <c r="B14" s="30"/>
+        <v>37</v>
+      </c>
+      <c r="B14" s="30">
+        <v>46276</v>
+      </c>
       <c r="C14" s="31"/>
       <c r="D14" s="32">
         <v>30</v>
@@ -4648,11 +4655,13 @@
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A15" s="63" t="str">
+      <c r="A15" s="63">
         <f>IF(ISBLANK(B15),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B15))</f>
-        <v/>
-      </c>
-      <c r="B15" s="34"/>
+        <v>37</v>
+      </c>
+      <c r="B15" s="34">
+        <v>46276</v>
+      </c>
       <c r="C15" s="35">
         <v>1</v>
       </c>
@@ -4674,11 +4683,13 @@
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A16" s="62" t="str">
+      <c r="A16" s="62">
         <f>IF(ISBLANK(B16),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B16))</f>
-        <v/>
-      </c>
-      <c r="B16" s="30"/>
+        <v>37</v>
+      </c>
+      <c r="B16" s="30">
+        <v>46276</v>
+      </c>
       <c r="C16" s="31"/>
       <c r="D16" s="32">
         <v>30</v>
@@ -4697,11 +4708,13 @@
       </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A17" s="63" t="str">
+      <c r="A17" s="63">
         <f>IF(ISBLANK(B17),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B17))</f>
-        <v/>
-      </c>
-      <c r="B17" s="34"/>
+        <v>37</v>
+      </c>
+      <c r="B17" s="34">
+        <v>46276</v>
+      </c>
       <c r="C17" s="35"/>
       <c r="D17" s="36">
         <v>30</v>
@@ -4720,11 +4733,13 @@
       </c>
     </row>
     <row r="18" spans="1:15" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A18" s="62" t="str">
+      <c r="A18" s="62">
         <f>IF(ISBLANK(B18),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B18))</f>
-        <v/>
-      </c>
-      <c r="B18" s="30"/>
+        <v>38</v>
+      </c>
+      <c r="B18" s="30">
+        <v>46283</v>
+      </c>
       <c r="C18" s="31">
         <v>1</v>
       </c>
@@ -4743,11 +4758,13 @@
       </c>
     </row>
     <row r="19" spans="1:15" ht="47.25" x14ac:dyDescent="0.25">
-      <c r="A19" s="63" t="str">
+      <c r="A19" s="63">
         <f>IF(ISBLANK(B19),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B19))</f>
-        <v/>
-      </c>
-      <c r="B19" s="34"/>
+        <v>38</v>
+      </c>
+      <c r="B19" s="34">
+        <v>46283</v>
+      </c>
       <c r="C19" s="35">
         <v>1</v>
       </c>
@@ -4766,11 +4783,13 @@
       </c>
     </row>
     <row r="20" spans="1:15" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A20" s="62" t="str">
+      <c r="A20" s="62">
         <f>IF(ISBLANK(B20),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B20))</f>
-        <v/>
-      </c>
-      <c r="B20" s="30"/>
+        <v>39</v>
+      </c>
+      <c r="B20" s="30">
+        <v>46288</v>
+      </c>
       <c r="C20" s="31">
         <v>1</v>
       </c>
@@ -4788,11 +4807,13 @@
       </c>
     </row>
     <row r="21" spans="1:15" ht="47.25" x14ac:dyDescent="0.25">
-      <c r="A21" s="63" t="str">
+      <c r="A21" s="63">
         <f>IF(ISBLANK(B21),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B21))</f>
-        <v/>
-      </c>
-      <c r="B21" s="34"/>
+        <v>39</v>
+      </c>
+      <c r="B21" s="34">
+        <v>46290</v>
+      </c>
       <c r="C21" s="35"/>
       <c r="D21" s="36">
         <v>30</v>
@@ -4806,11 +4827,13 @@
       <c r="G21" s="40"/>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A22" s="62" t="str">
+      <c r="A22" s="62">
         <f>IF(ISBLANK(B22),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B22))</f>
-        <v/>
-      </c>
-      <c r="B22" s="30"/>
+        <v>39</v>
+      </c>
+      <c r="B22" s="30">
+        <v>46290</v>
+      </c>
       <c r="C22" s="31"/>
       <c r="D22" s="32">
         <v>20</v>
@@ -4823,16 +4846,26 @@
       </c>
       <c r="G22" s="39"/>
     </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A23" s="63" t="str">
+    <row r="23" spans="1:15" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="A23" s="63">
         <f>IF(ISBLANK(B23),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B23))</f>
-        <v/>
-      </c>
-      <c r="B23" s="34"/>
-      <c r="C23" s="35"/>
-      <c r="D23" s="36"/>
-      <c r="E23" s="37"/>
-      <c r="F23" s="23"/>
+        <v>40</v>
+      </c>
+      <c r="B23" s="34">
+        <v>46297</v>
+      </c>
+      <c r="C23" s="35">
+        <v>2</v>
+      </c>
+      <c r="D23" s="36">
+        <v>30</v>
+      </c>
+      <c r="E23" s="37" t="s">
+        <v>16</v>
+      </c>
+      <c r="F23" s="23" t="s">
+        <v>49</v>
+      </c>
       <c r="G23" s="40"/>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.25">
@@ -11097,7 +11130,7 @@
       </c>
       <c r="G6" s="72">
         <f>SUM(A6:B6)/$C$11</f>
-        <v>9.0225563909774431E-2</v>
+        <v>7.3619631901840496E-2</v>
       </c>
       <c r="L6" s="51" t="str">
         <f>'Journal de travail'!M8</f>
@@ -11114,15 +11147,15 @@
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$C$7:$C$532)*60</f>
-        <v>240</v>
+        <v>360</v>
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$D$7:$D$532)</f>
-        <v>230</v>
+        <v>260</v>
       </c>
       <c r="C7">
         <f t="shared" si="0"/>
-        <v>470</v>
+        <v>620</v>
       </c>
       <c r="E7" s="73" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11130,11 +11163,11 @@
       </c>
       <c r="F7" s="74" t="str">
         <f t="shared" ref="F7:F11" si="1">QUOTIENT(SUM(A7:B7),60)&amp;" h "&amp;TEXT(MOD(SUM(A7:B7),60), "00")&amp;" min"</f>
-        <v>7 h 50 min</v>
+        <v>10 h 20 min</v>
       </c>
       <c r="G7" s="75">
         <f t="shared" ref="G7:G9" si="2">SUM(A7:B7)/$C$11</f>
-        <v>0.70676691729323304</v>
+        <v>0.76073619631901845</v>
       </c>
       <c r="L7" s="53" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11208,7 +11241,7 @@
       </c>
       <c r="G9" s="75">
         <f t="shared" si="2"/>
-        <v>0.20300751879699247</v>
+        <v>0.16564417177914109</v>
       </c>
       <c r="L9" s="55" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11260,26 +11293,26 @@
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11">
         <f>SUM(A6:A10)</f>
-        <v>360</v>
+        <v>480</v>
       </c>
       <c r="B11">
         <f>SUM(B6:B10)</f>
-        <v>305</v>
+        <v>335</v>
       </c>
       <c r="C11">
         <f>SUM(A11:B11)</f>
-        <v>665</v>
+        <v>815</v>
       </c>
       <c r="E11" s="81" t="s">
         <v>29</v>
       </c>
       <c r="F11" s="71" t="str">
         <f t="shared" si="1"/>
-        <v>11 h 05 min</v>
+        <v>13 h 35 min</v>
       </c>
       <c r="G11" s="82">
         <f>C11/C12</f>
-        <v>0.1259469696969697</v>
+        <v>0.15435606060606061</v>
       </c>
       <c r="L11" s="56" t="s">
         <v>29</v>

</xml_diff>

<commit_message>
feat(ShowStats) : On peut désormais afficher toutes les statistiques du jour :  nombre de place occupées, % du total, montant total payé, durée de stationnement actuel de tous les véhicules.
</commit_message>
<xml_diff>
--- a/fichiers/P_parking-jdt-HugoSchweizer.xlsx
+++ b/fichiers/P_parking-jdt-HugoSchweizer.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\P_parking\fichiers\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AB65B42-7C57-4C36-A188-02576AC76E7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E868C451-3371-4584-B346-521398E381EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="51">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -191,6 +191,10 @@
   </si>
   <si>
     <t>J'ai modifié le calcule du temps et le calcule du prix du ticket qui n'était pas du tout correcte, et j'ai aussi ajouté un prix de ticket minimum. L'affiche du ticket aussi à été modifié ainsi que les véhicules présents dans le parking quand on affiche le parking.</t>
+  </si>
+  <si>
+    <t>On peut désormais afficher toutes les statistiques du jour :  nombre de place occupées, 
+% du total, montant total payé, durée de stationnement actuel de tous les véhicules.</t>
   </si>
 </sst>
 </file>
@@ -1201,7 +1205,7 @@
                   <c:v>60</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>620</c:v>
+                  <c:v>650</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -2131,16 +2135,16 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>7.3619631901840496E-2</c:v>
+                  <c:v>7.1005917159763315E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.76073619631901845</c:v>
+                  <c:v>0.76923076923076927</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.16564417177914109</c:v>
+                  <c:v>0.15976331360946747</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -4378,7 +4382,7 @@
       <c r="B3" s="86"/>
       <c r="C3" s="67" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>14 heures 5 minutes</v>
+        <v>14 heures 35 minutes</v>
       </c>
       <c r="D3" s="17"/>
       <c r="E3" s="3"/>
@@ -4397,11 +4401,11 @@
       </c>
       <c r="D4" s="17">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>365</v>
+        <v>395</v>
       </c>
       <c r="E4" s="24">
         <f>SUM(C4:D4)</f>
-        <v>845</v>
+        <v>875</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -4868,16 +4872,24 @@
       </c>
       <c r="G23" s="40"/>
     </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A24" s="62" t="str">
+    <row r="24" spans="1:15" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A24" s="62">
         <f>IF(ISBLANK(B24),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B24))</f>
-        <v/>
-      </c>
-      <c r="B24" s="30"/>
+        <v>40</v>
+      </c>
+      <c r="B24" s="30">
+        <v>46297</v>
+      </c>
       <c r="C24" s="31"/>
-      <c r="D24" s="32"/>
-      <c r="E24" s="33"/>
-      <c r="F24" s="23"/>
+      <c r="D24" s="32">
+        <v>30</v>
+      </c>
+      <c r="E24" s="33" t="s">
+        <v>16</v>
+      </c>
+      <c r="F24" s="23" t="s">
+        <v>50</v>
+      </c>
       <c r="G24" s="39"/>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.25">
@@ -11130,7 +11142,7 @@
       </c>
       <c r="G6" s="72">
         <f>SUM(A6:B6)/$C$11</f>
-        <v>7.3619631901840496E-2</v>
+        <v>7.1005917159763315E-2</v>
       </c>
       <c r="L6" s="51" t="str">
         <f>'Journal de travail'!M8</f>
@@ -11151,11 +11163,11 @@
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$D$7:$D$532)</f>
-        <v>260</v>
+        <v>290</v>
       </c>
       <c r="C7">
         <f t="shared" si="0"/>
-        <v>620</v>
+        <v>650</v>
       </c>
       <c r="E7" s="73" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11163,11 +11175,11 @@
       </c>
       <c r="F7" s="74" t="str">
         <f t="shared" ref="F7:F11" si="1">QUOTIENT(SUM(A7:B7),60)&amp;" h "&amp;TEXT(MOD(SUM(A7:B7),60), "00")&amp;" min"</f>
-        <v>10 h 20 min</v>
+        <v>10 h 50 min</v>
       </c>
       <c r="G7" s="75">
         <f t="shared" ref="G7:G9" si="2">SUM(A7:B7)/$C$11</f>
-        <v>0.76073619631901845</v>
+        <v>0.76923076923076927</v>
       </c>
       <c r="L7" s="53" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11241,7 +11253,7 @@
       </c>
       <c r="G9" s="75">
         <f t="shared" si="2"/>
-        <v>0.16564417177914109</v>
+        <v>0.15976331360946747</v>
       </c>
       <c r="L9" s="55" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11297,22 +11309,22 @@
       </c>
       <c r="B11">
         <f>SUM(B6:B10)</f>
-        <v>335</v>
+        <v>365</v>
       </c>
       <c r="C11">
         <f>SUM(A11:B11)</f>
-        <v>815</v>
+        <v>845</v>
       </c>
       <c r="E11" s="81" t="s">
         <v>29</v>
       </c>
       <c r="F11" s="71" t="str">
         <f t="shared" si="1"/>
-        <v>13 h 35 min</v>
+        <v>14 h 05 min</v>
       </c>
       <c r="G11" s="82">
         <f>C11/C12</f>
-        <v>0.15435606060606061</v>
+        <v>0.16003787878787878</v>
       </c>
       <c r="L11" s="56" t="s">
         <v>29</v>
@@ -11351,12 +11363,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="4356f79f-5386-4bda-9d92-82d8bd7b074e" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3eb094ff-ec8d-44d8-be06-94ad3ec8832a">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -11561,20 +11575,21 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="4356f79f-5386-4bda-9d92-82d8bd7b074e" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3eb094ff-ec8d-44d8-be06-94ad3ec8832a">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="4356f79f-5386-4bda-9d92-82d8bd7b074e"/>
+    <ds:schemaRef ds:uri="3eb094ff-ec8d-44d8-be06-94ad3ec8832a"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -11599,12 +11614,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="4356f79f-5386-4bda-9d92-82d8bd7b074e"/>
-    <ds:schemaRef ds:uri="3eb094ff-ec8d-44d8-be06-94ad3ec8832a"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
feat(ShowTransactionHistory) : J'ai ajouté le faite de pouvoir voir toutes les transcations du jours : la plaque de la voiture, heure d'entrée, heure de sortie (si déjà sortie), temps passé dans le parking, prix du ticket (si déjà sortie). S'ils sont rentrés plusieurs fois dans le parking, ils s'afficheront plusieurs fois
</commit_message>
<xml_diff>
--- a/fichiers/P_parking-jdt-HugoSchweizer.xlsx
+++ b/fichiers/P_parking-jdt-HugoSchweizer.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\P_parking\fichiers\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\P_parking\fichiers\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E868C451-3371-4584-B346-521398E381EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23515E00-FB18-4833-81AF-2916E1026BF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal de travail" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="52">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -195,6 +195,9 @@
   <si>
     <t>On peut désormais afficher toutes les statistiques du jour :  nombre de place occupées, 
 % du total, montant total payé, durée de stationnement actuel de tous les véhicules.</t>
+  </si>
+  <si>
+    <t>J'ai ajouté le faite de pouvoir voir toutes les transcations du jours : la plaque de la voiture, heure d'entrée, heure de sortie (si déjà sortie), temps passé dans le parking, prix du ticket (si déjà sortie). S'ils sont rentrés plusieurs fois dans le parking, ils s'afficheront plusieurs fois</t>
   </si>
 </sst>
 </file>
@@ -957,7 +960,7 @@
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="fr-FR"/>
+  <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -1205,7 +1208,7 @@
                   <c:v>60</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>650</c:v>
+                  <c:v>710</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -1323,7 +1326,7 @@
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="fr-FR"/>
+  <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -1696,7 +1699,7 @@
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="fr-FR"/>
+  <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -2135,16 +2138,16 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>7.1005917159763315E-2</c:v>
+                  <c:v>6.6298342541436461E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.76923076923076927</c:v>
+                  <c:v>0.78453038674033149</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.15976331360946747</c:v>
+                  <c:v>0.14917127071823205</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -4330,7 +4333,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8FF2E8F1-C793-7E43-B3DE-C075053A97DA}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:O532"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.5" style="7" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11.875" style="1" customWidth="1"/>
@@ -4382,7 +4385,7 @@
       <c r="B3" s="86"/>
       <c r="C3" s="67" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>14 heures 35 minutes</v>
+        <v>15 heures 35 minutes</v>
       </c>
       <c r="D3" s="17"/>
       <c r="E3" s="3"/>
@@ -4397,7 +4400,7 @@
       <c r="B4" s="5"/>
       <c r="C4" s="17">
         <f>SUBTOTAL(9,$C$7:$C$531)*60</f>
-        <v>480</v>
+        <v>540</v>
       </c>
       <c r="D4" s="17">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
@@ -4405,7 +4408,7 @@
       </c>
       <c r="E4" s="24">
         <f>SUM(C4:D4)</f>
-        <v>875</v>
+        <v>935</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -4892,16 +4895,26 @@
       </c>
       <c r="G24" s="39"/>
     </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A25" s="63" t="str">
+    <row r="25" spans="1:15" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="A25" s="63">
         <f>IF(ISBLANK(B25),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B25))</f>
-        <v/>
-      </c>
-      <c r="B25" s="34"/>
-      <c r="C25" s="35"/>
-      <c r="D25" s="36"/>
-      <c r="E25" s="37"/>
-      <c r="F25" s="23"/>
+        <v>40</v>
+      </c>
+      <c r="B25" s="34">
+        <v>46298</v>
+      </c>
+      <c r="C25" s="35">
+        <v>1</v>
+      </c>
+      <c r="D25" s="36">
+        <v>0</v>
+      </c>
+      <c r="E25" s="37" t="s">
+        <v>16</v>
+      </c>
+      <c r="F25" s="23" t="s">
+        <v>51</v>
+      </c>
       <c r="G25" s="40"/>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.25">
@@ -11048,7 +11061,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D21D7432-C939-0D45-BAC2-A6A2196EA9C6}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A2:N13"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="3" width="10.875" hidden="1" customWidth="1"/>
     <col min="4" max="4" width="10.875" customWidth="1"/>
@@ -11142,7 +11155,7 @@
       </c>
       <c r="G6" s="72">
         <f>SUM(A6:B6)/$C$11</f>
-        <v>7.1005917159763315E-2</v>
+        <v>6.6298342541436461E-2</v>
       </c>
       <c r="L6" s="51" t="str">
         <f>'Journal de travail'!M8</f>
@@ -11159,7 +11172,7 @@
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$C$7:$C$532)*60</f>
-        <v>360</v>
+        <v>420</v>
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$D$7:$D$532)</f>
@@ -11167,7 +11180,7 @@
       </c>
       <c r="C7">
         <f t="shared" si="0"/>
-        <v>650</v>
+        <v>710</v>
       </c>
       <c r="E7" s="73" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11175,11 +11188,11 @@
       </c>
       <c r="F7" s="74" t="str">
         <f t="shared" ref="F7:F11" si="1">QUOTIENT(SUM(A7:B7),60)&amp;" h "&amp;TEXT(MOD(SUM(A7:B7),60), "00")&amp;" min"</f>
-        <v>10 h 50 min</v>
+        <v>11 h 50 min</v>
       </c>
       <c r="G7" s="75">
         <f t="shared" ref="G7:G9" si="2">SUM(A7:B7)/$C$11</f>
-        <v>0.76923076923076927</v>
+        <v>0.78453038674033149</v>
       </c>
       <c r="L7" s="53" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11253,7 +11266,7 @@
       </c>
       <c r="G9" s="75">
         <f t="shared" si="2"/>
-        <v>0.15976331360946747</v>
+        <v>0.14917127071823205</v>
       </c>
       <c r="L9" s="55" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11305,7 +11318,7 @@
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11">
         <f>SUM(A6:A10)</f>
-        <v>480</v>
+        <v>540</v>
       </c>
       <c r="B11">
         <f>SUM(B6:B10)</f>
@@ -11313,18 +11326,18 @@
       </c>
       <c r="C11">
         <f>SUM(A11:B11)</f>
-        <v>845</v>
+        <v>905</v>
       </c>
       <c r="E11" s="81" t="s">
         <v>29</v>
       </c>
       <c r="F11" s="71" t="str">
         <f t="shared" si="1"/>
-        <v>14 h 05 min</v>
+        <v>15 h 05 min</v>
       </c>
       <c r="G11" s="82">
         <f>C11/C12</f>
-        <v>0.16003787878787878</v>
+        <v>0.17140151515151514</v>
       </c>
       <c r="L11" s="56" t="s">
         <v>29</v>
@@ -11354,7 +11367,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67F31118-7D2C-C547-B9C9-EA2B04E048B8}">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <sheetProtection algorithmName="SHA-512" hashValue="hkKOZ8xr/Okjo/AJlNTtoGYYhES8sIn2fOpGKGGyPJqhNRzaMuj9V6Pke+VqLSypQTwaNPCt0dhRPEVp9CfBFA==" saltValue="lF/ApQWS3LBdJp0wgcNUcQ==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -11363,14 +11376,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="4356f79f-5386-4bda-9d92-82d8bd7b074e" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3eb094ff-ec8d-44d8-be06-94ad3ec8832a">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -11575,21 +11586,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="4356f79f-5386-4bda-9d92-82d8bd7b074e" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3eb094ff-ec8d-44d8-be06-94ad3ec8832a">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="4356f79f-5386-4bda-9d92-82d8bd7b074e"/>
-    <ds:schemaRef ds:uri="3eb094ff-ec8d-44d8-be06-94ad3ec8832a"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -11614,9 +11624,12 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="4356f79f-5386-4bda-9d92-82d8bd7b074e"/>
+    <ds:schemaRef ds:uri="3eb094ff-ec8d-44d8-be06-94ad3ec8832a"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
feat(Test unitaires) : J'ai ajouté les tests unitaires en les testant sur ma methode CheckLicensePlate
</commit_message>
<xml_diff>
--- a/fichiers/P_parking-jdt-HugoSchweizer.xlsx
+++ b/fichiers/P_parking-jdt-HugoSchweizer.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\P_parking\fichiers\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23515E00-FB18-4833-81AF-2916E1026BF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0DE00DC-2F60-4778-97D4-19223198D666}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="54">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -198,6 +198,12 @@
   </si>
   <si>
     <t>J'ai ajouté le faite de pouvoir voir toutes les transcations du jours : la plaque de la voiture, heure d'entrée, heure de sortie (si déjà sortie), temps passé dans le parking, prix du ticket (si déjà sortie). S'ils sont rentrés plusieurs fois dans le parking, ils s'afficheront plusieurs fois</t>
+  </si>
+  <si>
+    <t>J'ai ajouté les tests unitaires en testant sur ma methode "CheckLicensePlate"</t>
+  </si>
+  <si>
+    <t>à la maison</t>
   </si>
 </sst>
 </file>
@@ -1208,7 +1214,7 @@
                   <c:v>60</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>710</c:v>
+                  <c:v>740</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -2138,16 +2144,16 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>6.6298342541436461E-2</c:v>
+                  <c:v>6.4171122994652413E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.78453038674033149</c:v>
+                  <c:v>0.79144385026737973</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.14917127071823205</c:v>
+                  <c:v>0.14438502673796791</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -4385,7 +4391,7 @@
       <c r="B3" s="86"/>
       <c r="C3" s="67" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>15 heures 35 minutes</v>
+        <v>16 heures 5 minutes</v>
       </c>
       <c r="D3" s="17"/>
       <c r="E3" s="3"/>
@@ -4404,11 +4410,11 @@
       </c>
       <c r="D4" s="17">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>395</v>
+        <v>425</v>
       </c>
       <c r="E4" s="24">
         <f>SUM(C4:D4)</f>
-        <v>935</v>
+        <v>965</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -4915,19 +4921,31 @@
       <c r="F25" s="23" t="s">
         <v>51</v>
       </c>
-      <c r="G25" s="40"/>
+      <c r="G25" s="40" t="s">
+        <v>53</v>
+      </c>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A26" s="62" t="str">
+      <c r="A26" s="62">
         <f>IF(ISBLANK(B26),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B26))</f>
-        <v/>
-      </c>
-      <c r="B26" s="30"/>
+        <v>40</v>
+      </c>
+      <c r="B26" s="30">
+        <v>46298</v>
+      </c>
       <c r="C26" s="31"/>
-      <c r="D26" s="32"/>
-      <c r="E26" s="33"/>
-      <c r="F26" s="23"/>
-      <c r="G26" s="39"/>
+      <c r="D26" s="32">
+        <v>30</v>
+      </c>
+      <c r="E26" s="33" t="s">
+        <v>16</v>
+      </c>
+      <c r="F26" s="23" t="s">
+        <v>52</v>
+      </c>
+      <c r="G26" s="39" t="s">
+        <v>53</v>
+      </c>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A27" s="63" t="str">
@@ -11155,7 +11173,7 @@
       </c>
       <c r="G6" s="72">
         <f>SUM(A6:B6)/$C$11</f>
-        <v>6.6298342541436461E-2</v>
+        <v>6.4171122994652413E-2</v>
       </c>
       <c r="L6" s="51" t="str">
         <f>'Journal de travail'!M8</f>
@@ -11176,11 +11194,11 @@
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$D$7:$D$532)</f>
-        <v>290</v>
+        <v>320</v>
       </c>
       <c r="C7">
         <f t="shared" si="0"/>
-        <v>710</v>
+        <v>740</v>
       </c>
       <c r="E7" s="73" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11188,11 +11206,11 @@
       </c>
       <c r="F7" s="74" t="str">
         <f t="shared" ref="F7:F11" si="1">QUOTIENT(SUM(A7:B7),60)&amp;" h "&amp;TEXT(MOD(SUM(A7:B7),60), "00")&amp;" min"</f>
-        <v>11 h 50 min</v>
+        <v>12 h 20 min</v>
       </c>
       <c r="G7" s="75">
         <f t="shared" ref="G7:G9" si="2">SUM(A7:B7)/$C$11</f>
-        <v>0.78453038674033149</v>
+        <v>0.79144385026737973</v>
       </c>
       <c r="L7" s="53" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11266,7 +11284,7 @@
       </c>
       <c r="G9" s="75">
         <f t="shared" si="2"/>
-        <v>0.14917127071823205</v>
+        <v>0.14438502673796791</v>
       </c>
       <c r="L9" s="55" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11322,22 +11340,22 @@
       </c>
       <c r="B11">
         <f>SUM(B6:B10)</f>
-        <v>365</v>
+        <v>395</v>
       </c>
       <c r="C11">
         <f>SUM(A11:B11)</f>
-        <v>905</v>
+        <v>935</v>
       </c>
       <c r="E11" s="81" t="s">
         <v>29</v>
       </c>
       <c r="F11" s="71" t="str">
         <f t="shared" si="1"/>
-        <v>15 h 05 min</v>
+        <v>15 h 35 min</v>
       </c>
       <c r="G11" s="82">
         <f>C11/C12</f>
-        <v>0.17140151515151514</v>
+        <v>0.17708333333333334</v>
       </c>
       <c r="L11" s="56" t="s">
         <v>29</v>
@@ -11376,12 +11394,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="4356f79f-5386-4bda-9d92-82d8bd7b074e" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3eb094ff-ec8d-44d8-be06-94ad3ec8832a">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -11586,20 +11606,21 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="4356f79f-5386-4bda-9d92-82d8bd7b074e" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3eb094ff-ec8d-44d8-be06-94ad3ec8832a">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="4356f79f-5386-4bda-9d92-82d8bd7b074e"/>
+    <ds:schemaRef ds:uri="3eb094ff-ec8d-44d8-be06-94ad3ec8832a"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -11624,12 +11645,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="4356f79f-5386-4bda-9d92-82d8bd7b074e"/>
-    <ds:schemaRef ds:uri="3eb094ff-ec8d-44d8-be06-94ad3ec8832a"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
feat(Tests Unitaires) : ajouts de deux autres tests unitaires sur la methode CheckLicensePlate
</commit_message>
<xml_diff>
--- a/fichiers/P_parking-jdt-HugoSchweizer.xlsx
+++ b/fichiers/P_parking-jdt-HugoSchweizer.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\P_parking\fichiers\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0DE00DC-2F60-4778-97D4-19223198D666}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FD88289-29C4-44D0-8876-C292A5AE0091}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="55">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -204,6 +204,9 @@
   </si>
   <si>
     <t>à la maison</t>
+  </si>
+  <si>
+    <t>J'ai ajouté deux autres tests unitaires sur la methode "CheckLicensePlate"</t>
   </si>
 </sst>
 </file>
@@ -1214,7 +1217,7 @@
                   <c:v>60</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>740</c:v>
+                  <c:v>760</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -2144,16 +2147,16 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>6.4171122994652413E-2</c:v>
+                  <c:v>6.2827225130890049E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.79144385026737973</c:v>
+                  <c:v>0.79581151832460728</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.14438502673796791</c:v>
+                  <c:v>0.14136125654450263</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -4391,7 +4394,7 @@
       <c r="B3" s="86"/>
       <c r="C3" s="67" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>16 heures 5 minutes</v>
+        <v>16 heures 25 minutes</v>
       </c>
       <c r="D3" s="17"/>
       <c r="E3" s="3"/>
@@ -4410,11 +4413,11 @@
       </c>
       <c r="D4" s="17">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>425</v>
+        <v>445</v>
       </c>
       <c r="E4" s="24">
         <f>SUM(C4:D4)</f>
-        <v>965</v>
+        <v>985</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -4948,16 +4951,26 @@
       </c>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A27" s="63" t="str">
+      <c r="A27" s="63">
         <f>IF(ISBLANK(B27),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B27))</f>
-        <v/>
-      </c>
-      <c r="B27" s="34"/>
+        <v>40</v>
+      </c>
+      <c r="B27" s="34">
+        <v>46299</v>
+      </c>
       <c r="C27" s="35"/>
-      <c r="D27" s="36"/>
-      <c r="E27" s="37"/>
-      <c r="F27" s="23"/>
-      <c r="G27" s="40"/>
+      <c r="D27" s="36">
+        <v>20</v>
+      </c>
+      <c r="E27" s="37" t="s">
+        <v>16</v>
+      </c>
+      <c r="F27" s="23" t="s">
+        <v>54</v>
+      </c>
+      <c r="G27" s="40" t="s">
+        <v>53</v>
+      </c>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A28" s="62" t="str">
@@ -11173,7 +11186,7 @@
       </c>
       <c r="G6" s="72">
         <f>SUM(A6:B6)/$C$11</f>
-        <v>6.4171122994652413E-2</v>
+        <v>6.2827225130890049E-2</v>
       </c>
       <c r="L6" s="51" t="str">
         <f>'Journal de travail'!M8</f>
@@ -11194,11 +11207,11 @@
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$D$7:$D$532)</f>
-        <v>320</v>
+        <v>340</v>
       </c>
       <c r="C7">
         <f t="shared" si="0"/>
-        <v>740</v>
+        <v>760</v>
       </c>
       <c r="E7" s="73" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11206,11 +11219,11 @@
       </c>
       <c r="F7" s="74" t="str">
         <f t="shared" ref="F7:F11" si="1">QUOTIENT(SUM(A7:B7),60)&amp;" h "&amp;TEXT(MOD(SUM(A7:B7),60), "00")&amp;" min"</f>
-        <v>12 h 20 min</v>
+        <v>12 h 40 min</v>
       </c>
       <c r="G7" s="75">
         <f t="shared" ref="G7:G9" si="2">SUM(A7:B7)/$C$11</f>
-        <v>0.79144385026737973</v>
+        <v>0.79581151832460728</v>
       </c>
       <c r="L7" s="53" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11284,7 +11297,7 @@
       </c>
       <c r="G9" s="75">
         <f t="shared" si="2"/>
-        <v>0.14438502673796791</v>
+        <v>0.14136125654450263</v>
       </c>
       <c r="L9" s="55" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11340,22 +11353,22 @@
       </c>
       <c r="B11">
         <f>SUM(B6:B10)</f>
-        <v>395</v>
+        <v>415</v>
       </c>
       <c r="C11">
         <f>SUM(A11:B11)</f>
-        <v>935</v>
+        <v>955</v>
       </c>
       <c r="E11" s="81" t="s">
         <v>29</v>
       </c>
       <c r="F11" s="71" t="str">
         <f t="shared" si="1"/>
-        <v>15 h 35 min</v>
+        <v>15 h 55 min</v>
       </c>
       <c r="G11" s="82">
         <f>C11/C12</f>
-        <v>0.17708333333333334</v>
+        <v>0.18087121212121213</v>
       </c>
       <c r="L11" s="56" t="s">
         <v>29</v>
@@ -11394,14 +11407,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="4356f79f-5386-4bda-9d92-82d8bd7b074e" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3eb094ff-ec8d-44d8-be06-94ad3ec8832a">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -11606,21 +11617,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="4356f79f-5386-4bda-9d92-82d8bd7b074e" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3eb094ff-ec8d-44d8-be06-94ad3ec8832a">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="4356f79f-5386-4bda-9d92-82d8bd7b074e"/>
-    <ds:schemaRef ds:uri="3eb094ff-ec8d-44d8-be06-94ad3ec8832a"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -11645,9 +11655,12 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="4356f79f-5386-4bda-9d92-82d8bd7b074e"/>
+    <ds:schemaRef ds:uri="3eb094ff-ec8d-44d8-be06-94ad3ec8832a"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
chore() : ancement dans le rapport du projet et commenatires du code ajouté
</commit_message>
<xml_diff>
--- a/fichiers/P_parking-jdt-HugoSchweizer.xlsx
+++ b/fichiers/P_parking-jdt-HugoSchweizer.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\P_parking\fichiers\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FD88289-29C4-44D0-8876-C292A5AE0091}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0DF1B56-9057-4E0A-A1D0-1D38F96C3B9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="56">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -207,6 +207,9 @@
   </si>
   <si>
     <t>J'ai ajouté deux autres tests unitaires sur la methode "CheckLicensePlate"</t>
+  </si>
+  <si>
+    <t>J'ai avancé dans le rapport du projet et en partie commanté le code</t>
   </si>
 </sst>
 </file>
@@ -1223,7 +1226,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>135</c:v>
+                  <c:v>195</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -2147,16 +2150,16 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>6.2827225130890049E-2</c:v>
+                  <c:v>5.9113300492610835E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.79581151832460728</c:v>
+                  <c:v>0.74876847290640391</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.14136125654450263</c:v>
+                  <c:v>0.19211822660098521</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -4394,7 +4397,7 @@
       <c r="B3" s="86"/>
       <c r="C3" s="67" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>16 heures 25 minutes</v>
+        <v>17 heures 25 minutes</v>
       </c>
       <c r="D3" s="17"/>
       <c r="E3" s="3"/>
@@ -4409,7 +4412,7 @@
       <c r="B4" s="5"/>
       <c r="C4" s="17">
         <f>SUBTOTAL(9,$C$7:$C$531)*60</f>
-        <v>540</v>
+        <v>600</v>
       </c>
       <c r="D4" s="17">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
@@ -4417,7 +4420,7 @@
       </c>
       <c r="E4" s="24">
         <f>SUM(C4:D4)</f>
-        <v>985</v>
+        <v>1045</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -4973,16 +4976,26 @@
       </c>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A28" s="62" t="str">
+      <c r="A28" s="62">
         <f>IF(ISBLANK(B28),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B28))</f>
-        <v/>
-      </c>
-      <c r="B28" s="30"/>
-      <c r="C28" s="31"/>
+        <v>40</v>
+      </c>
+      <c r="B28" s="30">
+        <v>46299</v>
+      </c>
+      <c r="C28" s="31">
+        <v>1</v>
+      </c>
       <c r="D28" s="32"/>
-      <c r="E28" s="33"/>
-      <c r="F28" s="22"/>
-      <c r="G28" s="39"/>
+      <c r="E28" s="33" t="s">
+        <v>17</v>
+      </c>
+      <c r="F28" s="22" t="s">
+        <v>55</v>
+      </c>
+      <c r="G28" s="39" t="s">
+        <v>53</v>
+      </c>
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A29" s="63" t="str">
@@ -11186,7 +11199,7 @@
       </c>
       <c r="G6" s="72">
         <f>SUM(A6:B6)/$C$11</f>
-        <v>6.2827225130890049E-2</v>
+        <v>5.9113300492610835E-2</v>
       </c>
       <c r="L6" s="51" t="str">
         <f>'Journal de travail'!M8</f>
@@ -11223,7 +11236,7 @@
       </c>
       <c r="G7" s="75">
         <f t="shared" ref="G7:G9" si="2">SUM(A7:B7)/$C$11</f>
-        <v>0.79581151832460728</v>
+        <v>0.74876847290640391</v>
       </c>
       <c r="L7" s="53" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11277,7 +11290,7 @@
     <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E9,'Journal de travail'!$C$7:$C$532)*60</f>
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="B9">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E9,'Journal de travail'!$D$7:$D$532)</f>
@@ -11285,7 +11298,7 @@
       </c>
       <c r="C9">
         <f t="shared" si="0"/>
-        <v>135</v>
+        <v>195</v>
       </c>
       <c r="E9" s="77" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11293,11 +11306,11 @@
       </c>
       <c r="F9" s="74" t="str">
         <f t="shared" si="1"/>
-        <v>2 h 15 min</v>
+        <v>3 h 15 min</v>
       </c>
       <c r="G9" s="75">
         <f t="shared" si="2"/>
-        <v>0.14136125654450263</v>
+        <v>0.19211822660098521</v>
       </c>
       <c r="L9" s="55" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11349,7 +11362,7 @@
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11">
         <f>SUM(A6:A10)</f>
-        <v>540</v>
+        <v>600</v>
       </c>
       <c r="B11">
         <f>SUM(B6:B10)</f>
@@ -11357,18 +11370,18 @@
       </c>
       <c r="C11">
         <f>SUM(A11:B11)</f>
-        <v>955</v>
+        <v>1015</v>
       </c>
       <c r="E11" s="81" t="s">
         <v>29</v>
       </c>
       <c r="F11" s="71" t="str">
         <f t="shared" si="1"/>
-        <v>15 h 55 min</v>
+        <v>16 h 55 min</v>
       </c>
       <c r="G11" s="82">
         <f>C11/C12</f>
-        <v>0.18087121212121213</v>
+        <v>0.19223484848484848</v>
       </c>
       <c r="L11" s="56" t="s">
         <v>29</v>
@@ -11407,12 +11420,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="4356f79f-5386-4bda-9d92-82d8bd7b074e" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3eb094ff-ec8d-44d8-be06-94ad3ec8832a">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -11617,20 +11632,21 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="4356f79f-5386-4bda-9d92-82d8bd7b074e" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3eb094ff-ec8d-44d8-be06-94ad3ec8832a">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="4356f79f-5386-4bda-9d92-82d8bd7b074e"/>
+    <ds:schemaRef ds:uri="3eb094ff-ec8d-44d8-be06-94ad3ec8832a"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -11655,12 +11671,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="4356f79f-5386-4bda-9d92-82d8bd7b074e"/>
-    <ds:schemaRef ds:uri="3eb094ff-ec8d-44d8-be06-94ad3ec8832a"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Doc(Word) : J'ai fini de remplire mon word. En faisant les derniers chapitres (Conception, Utilisation de l'IA, Bilan déroulement, Bilan produit, Conclusion)
</commit_message>
<xml_diff>
--- a/fichiers/P_parking-jdt-HugoSchweizer.xlsx
+++ b/fichiers/P_parking-jdt-HugoSchweizer.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\P_parking\fichiers\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\P_parking\fichiers\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0DF1B56-9057-4E0A-A1D0-1D38F96C3B9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A590C98D-83D3-47B6-A038-E91070064EBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal de travail" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="57">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -210,6 +210,9 @@
   </si>
   <si>
     <t>J'ai avancé dans le rapport du projet et en partie commanté le code</t>
+  </si>
+  <si>
+    <t>J'ai fini de remplire mon word. En faisant les derniers chapitres (Conception, Utilisation de l'IA, Bilan déroulement, Bilan produit, Conclusion)</t>
   </si>
 </sst>
 </file>
@@ -972,7 +975,7 @@
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
+  <c:lang val="fr-FR"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -1226,7 +1229,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>195</c:v>
+                  <c:v>375</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -1338,7 +1341,7 @@
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
+  <c:lang val="fr-FR"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -1711,7 +1714,7 @@
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
+  <c:lang val="fr-FR"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -2150,16 +2153,16 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>5.9113300492610835E-2</c:v>
+                  <c:v>5.0209205020920501E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.74876847290640391</c:v>
+                  <c:v>0.63598326359832635</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.19211822660098521</c:v>
+                  <c:v>0.31380753138075312</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -4345,7 +4348,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8FF2E8F1-C793-7E43-B3DE-C075053A97DA}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:O532"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.5" style="7" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11.875" style="1" customWidth="1"/>
@@ -4397,7 +4400,7 @@
       <c r="B3" s="86"/>
       <c r="C3" s="67" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>17 heures 25 minutes</v>
+        <v>20 heures 25 minutes</v>
       </c>
       <c r="D3" s="17"/>
       <c r="E3" s="3"/>
@@ -4412,7 +4415,7 @@
       <c r="B4" s="5"/>
       <c r="C4" s="17">
         <f>SUBTOTAL(9,$C$7:$C$531)*60</f>
-        <v>600</v>
+        <v>780</v>
       </c>
       <c r="D4" s="17">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
@@ -4420,7 +4423,7 @@
       </c>
       <c r="E4" s="24">
         <f>SUM(C4:D4)</f>
-        <v>1045</v>
+        <v>1225</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -5009,16 +5012,24 @@
       <c r="F29" s="22"/>
       <c r="G29" s="40"/>
     </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A30" s="62" t="str">
+    <row r="30" spans="1:15" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A30" s="62">
         <f>IF(ISBLANK(B30),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B30))</f>
-        <v/>
-      </c>
-      <c r="B30" s="30"/>
-      <c r="C30" s="31"/>
+        <v>41</v>
+      </c>
+      <c r="B30" s="30">
+        <v>46300</v>
+      </c>
+      <c r="C30" s="31">
+        <v>3</v>
+      </c>
       <c r="D30" s="32"/>
-      <c r="E30" s="33"/>
-      <c r="F30" s="23"/>
+      <c r="E30" s="33" t="s">
+        <v>17</v>
+      </c>
+      <c r="F30" s="23" t="s">
+        <v>56</v>
+      </c>
       <c r="G30" s="39"/>
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.25">
@@ -11105,7 +11116,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D21D7432-C939-0D45-BAC2-A6A2196EA9C6}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A2:N13"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="3" width="10.875" hidden="1" customWidth="1"/>
     <col min="4" max="4" width="10.875" customWidth="1"/>
@@ -11199,7 +11210,7 @@
       </c>
       <c r="G6" s="72">
         <f>SUM(A6:B6)/$C$11</f>
-        <v>5.9113300492610835E-2</v>
+        <v>5.0209205020920501E-2</v>
       </c>
       <c r="L6" s="51" t="str">
         <f>'Journal de travail'!M8</f>
@@ -11236,7 +11247,7 @@
       </c>
       <c r="G7" s="75">
         <f t="shared" ref="G7:G9" si="2">SUM(A7:B7)/$C$11</f>
-        <v>0.74876847290640391</v>
+        <v>0.63598326359832635</v>
       </c>
       <c r="L7" s="53" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11290,7 +11301,7 @@
     <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E9,'Journal de travail'!$C$7:$C$532)*60</f>
-        <v>120</v>
+        <v>300</v>
       </c>
       <c r="B9">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E9,'Journal de travail'!$D$7:$D$532)</f>
@@ -11298,7 +11309,7 @@
       </c>
       <c r="C9">
         <f t="shared" si="0"/>
-        <v>195</v>
+        <v>375</v>
       </c>
       <c r="E9" s="77" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11306,11 +11317,11 @@
       </c>
       <c r="F9" s="74" t="str">
         <f t="shared" si="1"/>
-        <v>3 h 15 min</v>
+        <v>6 h 15 min</v>
       </c>
       <c r="G9" s="75">
         <f t="shared" si="2"/>
-        <v>0.19211822660098521</v>
+        <v>0.31380753138075312</v>
       </c>
       <c r="L9" s="55" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11362,7 +11373,7 @@
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11">
         <f>SUM(A6:A10)</f>
-        <v>600</v>
+        <v>780</v>
       </c>
       <c r="B11">
         <f>SUM(B6:B10)</f>
@@ -11370,18 +11381,18 @@
       </c>
       <c r="C11">
         <f>SUM(A11:B11)</f>
-        <v>1015</v>
+        <v>1195</v>
       </c>
       <c r="E11" s="81" t="s">
         <v>29</v>
       </c>
       <c r="F11" s="71" t="str">
         <f t="shared" si="1"/>
-        <v>16 h 55 min</v>
+        <v>19 h 55 min</v>
       </c>
       <c r="G11" s="82">
         <f>C11/C12</f>
-        <v>0.19223484848484848</v>
+        <v>0.22632575757575757</v>
       </c>
       <c r="L11" s="56" t="s">
         <v>29</v>
@@ -11411,7 +11422,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67F31118-7D2C-C547-B9C9-EA2B04E048B8}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <sheetProtection algorithmName="SHA-512" hashValue="hkKOZ8xr/Okjo/AJlNTtoGYYhES8sIn2fOpGKGGyPJqhNRzaMuj9V6Pke+VqLSypQTwaNPCt0dhRPEVp9CfBFA==" saltValue="lF/ApQWS3LBdJp0wgcNUcQ==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -11420,14 +11431,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="4356f79f-5386-4bda-9d92-82d8bd7b074e" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3eb094ff-ec8d-44d8-be06-94ad3ec8832a">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -11632,21 +11641,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="4356f79f-5386-4bda-9d92-82d8bd7b074e" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3eb094ff-ec8d-44d8-be06-94ad3ec8832a">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="4356f79f-5386-4bda-9d92-82d8bd7b074e"/>
-    <ds:schemaRef ds:uri="3eb094ff-ec8d-44d8-be06-94ad3ec8832a"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -11671,9 +11679,12 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="4356f79f-5386-4bda-9d92-82d8bd7b074e"/>
+    <ds:schemaRef ds:uri="3eb094ff-ec8d-44d8-be06-94ad3ec8832a"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Doc(Commentaires) : Finalisation des commentaires du code
</commit_message>
<xml_diff>
--- a/fichiers/P_parking-jdt-HugoSchweizer.xlsx
+++ b/fichiers/P_parking-jdt-HugoSchweizer.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\P_parking\fichiers\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A590C98D-83D3-47B6-A038-E91070064EBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73D64694-56FA-40D0-BD49-142C70EF993B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="58">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -213,6 +213,9 @@
   </si>
   <si>
     <t>J'ai fini de remplire mon word. En faisant les derniers chapitres (Conception, Utilisation de l'IA, Bilan déroulement, Bilan produit, Conclusion)</t>
+  </si>
+  <si>
+    <t>Finalisation des commentaires du code</t>
   </si>
 </sst>
 </file>
@@ -1229,7 +1232,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>375</c:v>
+                  <c:v>405</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -2153,16 +2156,16 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>5.0209205020920501E-2</c:v>
+                  <c:v>4.8979591836734691E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.63598326359832635</c:v>
+                  <c:v>0.62040816326530612</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.31380753138075312</c:v>
+                  <c:v>0.33061224489795921</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -4400,7 +4403,7 @@
       <c r="B3" s="86"/>
       <c r="C3" s="67" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>20 heures 25 minutes</v>
+        <v>20 heures 55 minutes</v>
       </c>
       <c r="D3" s="17"/>
       <c r="E3" s="3"/>
@@ -4419,11 +4422,11 @@
       </c>
       <c r="D4" s="17">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>445</v>
+        <v>475</v>
       </c>
       <c r="E4" s="24">
         <f>SUM(C4:D4)</f>
-        <v>1225</v>
+        <v>1255</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -4989,7 +4992,9 @@
       <c r="C28" s="31">
         <v>1</v>
       </c>
-      <c r="D28" s="32"/>
+      <c r="D28" s="32">
+        <v>0</v>
+      </c>
       <c r="E28" s="33" t="s">
         <v>17</v>
       </c>
@@ -5023,7 +5028,9 @@
       <c r="C30" s="31">
         <v>3</v>
       </c>
-      <c r="D30" s="32"/>
+      <c r="D30" s="32">
+        <v>0</v>
+      </c>
       <c r="E30" s="33" t="s">
         <v>17</v>
       </c>
@@ -5033,15 +5040,23 @@
       <c r="G30" s="39"/>
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A31" s="63" t="str">
+      <c r="A31" s="63">
         <f>IF(ISBLANK(B31),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B31))</f>
-        <v/>
-      </c>
-      <c r="B31" s="34"/>
+        <v>41</v>
+      </c>
+      <c r="B31" s="34">
+        <v>46300</v>
+      </c>
       <c r="C31" s="35"/>
-      <c r="D31" s="36"/>
-      <c r="E31" s="37"/>
-      <c r="F31" s="22"/>
+      <c r="D31" s="36">
+        <v>30</v>
+      </c>
+      <c r="E31" s="37" t="s">
+        <v>17</v>
+      </c>
+      <c r="F31" s="22" t="s">
+        <v>57</v>
+      </c>
       <c r="G31" s="40"/>
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.25">
@@ -11210,7 +11225,7 @@
       </c>
       <c r="G6" s="72">
         <f>SUM(A6:B6)/$C$11</f>
-        <v>5.0209205020920501E-2</v>
+        <v>4.8979591836734691E-2</v>
       </c>
       <c r="L6" s="51" t="str">
         <f>'Journal de travail'!M8</f>
@@ -11247,7 +11262,7 @@
       </c>
       <c r="G7" s="75">
         <f t="shared" ref="G7:G9" si="2">SUM(A7:B7)/$C$11</f>
-        <v>0.63598326359832635</v>
+        <v>0.62040816326530612</v>
       </c>
       <c r="L7" s="53" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11305,11 +11320,11 @@
       </c>
       <c r="B9">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E9,'Journal de travail'!$D$7:$D$532)</f>
-        <v>75</v>
+        <v>105</v>
       </c>
       <c r="C9">
         <f t="shared" si="0"/>
-        <v>375</v>
+        <v>405</v>
       </c>
       <c r="E9" s="77" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11317,11 +11332,11 @@
       </c>
       <c r="F9" s="74" t="str">
         <f t="shared" si="1"/>
-        <v>6 h 15 min</v>
+        <v>6 h 45 min</v>
       </c>
       <c r="G9" s="75">
         <f t="shared" si="2"/>
-        <v>0.31380753138075312</v>
+        <v>0.33061224489795921</v>
       </c>
       <c r="L9" s="55" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11377,22 +11392,22 @@
       </c>
       <c r="B11">
         <f>SUM(B6:B10)</f>
-        <v>415</v>
+        <v>445</v>
       </c>
       <c r="C11">
         <f>SUM(A11:B11)</f>
-        <v>1195</v>
+        <v>1225</v>
       </c>
       <c r="E11" s="81" t="s">
         <v>29</v>
       </c>
       <c r="F11" s="71" t="str">
         <f t="shared" si="1"/>
-        <v>19 h 55 min</v>
+        <v>20 h 25 min</v>
       </c>
       <c r="G11" s="82">
         <f>C11/C12</f>
-        <v>0.22632575757575757</v>
+        <v>0.23200757575757575</v>
       </c>
       <c r="L11" s="56" t="s">
         <v>29</v>
@@ -11431,12 +11446,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="4356f79f-5386-4bda-9d92-82d8bd7b074e" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3eb094ff-ec8d-44d8-be06-94ad3ec8832a">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -11641,20 +11658,21 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="4356f79f-5386-4bda-9d92-82d8bd7b074e" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3eb094ff-ec8d-44d8-be06-94ad3ec8832a">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="4356f79f-5386-4bda-9d92-82d8bd7b074e"/>
+    <ds:schemaRef ds:uri="3eb094ff-ec8d-44d8-be06-94ad3ec8832a"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -11679,12 +11697,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="4356f79f-5386-4bda-9d92-82d8bd7b074e"/>
-    <ds:schemaRef ds:uri="3eb094ff-ec8d-44d8-be06-94ad3ec8832a"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
chore() : Modification des commentaires avec les SUMMARY et les RETURNS pour les classes et les méthodes. Aussi modification du projet Test et modification des nom des méthodes de tests. Modification de la section test du rapport
</commit_message>
<xml_diff>
--- a/fichiers/P_parking-jdt-HugoSchweizer.xlsx
+++ b/fichiers/P_parking-jdt-HugoSchweizer.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\P_parking\fichiers\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73D64694-56FA-40D0-BD49-142C70EF993B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46D0D849-76F1-47D6-95F1-96C6F6B08156}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="59">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -216,6 +216,9 @@
   </si>
   <si>
     <t>Finalisation des commentaires du code</t>
+  </si>
+  <si>
+    <t>Modification des commentaires avec les SUMMARY et les RETURNS pour les classes et les méthodes. Aussi modification du projet Test et modification des nom des méthodes de tests. Modification de la section test du rapport</t>
   </si>
 </sst>
 </file>
@@ -1226,7 +1229,7 @@
                   <c:v>60</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>760</c:v>
+                  <c:v>820</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -2156,16 +2159,16 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>4.8979591836734691E-2</c:v>
+                  <c:v>4.6692607003891051E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.62040816326530612</c:v>
+                  <c:v>0.63813229571984431</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.33061224489795921</c:v>
+                  <c:v>0.31517509727626458</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -4403,7 +4406,7 @@
       <c r="B3" s="86"/>
       <c r="C3" s="67" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>20 heures 55 minutes</v>
+        <v>21 heures 55 minutes</v>
       </c>
       <c r="D3" s="17"/>
       <c r="E3" s="3"/>
@@ -4418,7 +4421,7 @@
       <c r="B4" s="5"/>
       <c r="C4" s="17">
         <f>SUBTOTAL(9,$C$7:$C$531)*60</f>
-        <v>780</v>
+        <v>840</v>
       </c>
       <c r="D4" s="17">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
@@ -4426,7 +4429,7 @@
       </c>
       <c r="E4" s="24">
         <f>SUM(C4:D4)</f>
-        <v>1255</v>
+        <v>1315</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -5059,16 +5062,26 @@
       </c>
       <c r="G31" s="40"/>
     </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A32" s="62" t="str">
+    <row r="32" spans="1:15" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="A32" s="62">
         <f>IF(ISBLANK(B32),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B32))</f>
-        <v/>
-      </c>
-      <c r="B32" s="30"/>
-      <c r="C32" s="31"/>
-      <c r="D32" s="32"/>
-      <c r="E32" s="33"/>
-      <c r="F32" s="23"/>
+        <v>41</v>
+      </c>
+      <c r="B32" s="30">
+        <v>46300</v>
+      </c>
+      <c r="C32" s="31">
+        <v>1</v>
+      </c>
+      <c r="D32" s="32">
+        <v>0</v>
+      </c>
+      <c r="E32" s="33" t="s">
+        <v>16</v>
+      </c>
+      <c r="F32" s="23" t="s">
+        <v>58</v>
+      </c>
       <c r="G32" s="39"/>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
@@ -11225,7 +11238,7 @@
       </c>
       <c r="G6" s="72">
         <f>SUM(A6:B6)/$C$11</f>
-        <v>4.8979591836734691E-2</v>
+        <v>4.6692607003891051E-2</v>
       </c>
       <c r="L6" s="51" t="str">
         <f>'Journal de travail'!M8</f>
@@ -11242,7 +11255,7 @@
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$C$7:$C$532)*60</f>
-        <v>420</v>
+        <v>480</v>
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$D$7:$D$532)</f>
@@ -11250,7 +11263,7 @@
       </c>
       <c r="C7">
         <f t="shared" si="0"/>
-        <v>760</v>
+        <v>820</v>
       </c>
       <c r="E7" s="73" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11258,11 +11271,11 @@
       </c>
       <c r="F7" s="74" t="str">
         <f t="shared" ref="F7:F11" si="1">QUOTIENT(SUM(A7:B7),60)&amp;" h "&amp;TEXT(MOD(SUM(A7:B7),60), "00")&amp;" min"</f>
-        <v>12 h 40 min</v>
+        <v>13 h 40 min</v>
       </c>
       <c r="G7" s="75">
         <f t="shared" ref="G7:G9" si="2">SUM(A7:B7)/$C$11</f>
-        <v>0.62040816326530612</v>
+        <v>0.63813229571984431</v>
       </c>
       <c r="L7" s="53" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11336,7 +11349,7 @@
       </c>
       <c r="G9" s="75">
         <f t="shared" si="2"/>
-        <v>0.33061224489795921</v>
+        <v>0.31517509727626458</v>
       </c>
       <c r="L9" s="55" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11388,7 +11401,7 @@
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11">
         <f>SUM(A6:A10)</f>
-        <v>780</v>
+        <v>840</v>
       </c>
       <c r="B11">
         <f>SUM(B6:B10)</f>
@@ -11396,18 +11409,18 @@
       </c>
       <c r="C11">
         <f>SUM(A11:B11)</f>
-        <v>1225</v>
+        <v>1285</v>
       </c>
       <c r="E11" s="81" t="s">
         <v>29</v>
       </c>
       <c r="F11" s="71" t="str">
         <f t="shared" si="1"/>
-        <v>20 h 25 min</v>
+        <v>21 h 25 min</v>
       </c>
       <c r="G11" s="82">
         <f>C11/C12</f>
-        <v>0.23200757575757575</v>
+        <v>0.24337121212121213</v>
       </c>
       <c r="L11" s="56" t="s">
         <v>29</v>
@@ -11446,14 +11459,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="4356f79f-5386-4bda-9d92-82d8bd7b074e" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3eb094ff-ec8d-44d8-be06-94ad3ec8832a">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -11658,21 +11669,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="4356f79f-5386-4bda-9d92-82d8bd7b074e" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3eb094ff-ec8d-44d8-be06-94ad3ec8832a">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="4356f79f-5386-4bda-9d92-82d8bd7b074e"/>
-    <ds:schemaRef ds:uri="3eb094ff-ec8d-44d8-be06-94ad3ec8832a"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -11697,9 +11707,12 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="4356f79f-5386-4bda-9d92-82d8bd7b074e"/>
+    <ds:schemaRef ds:uri="3eb094ff-ec8d-44d8-be06-94ad3ec8832a"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Doc() : Modifications de certains commentaires
</commit_message>
<xml_diff>
--- a/fichiers/P_parking-jdt-HugoSchweizer.xlsx
+++ b/fichiers/P_parking-jdt-HugoSchweizer.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\P_parking\fichiers\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46D0D849-76F1-47D6-95F1-96C6F6B08156}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B75835B-DC62-4A41-A425-82978D5DC5F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="60">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -219,6 +219,9 @@
   </si>
   <si>
     <t>Modification des commentaires avec les SUMMARY et les RETURNS pour les classes et les méthodes. Aussi modification du projet Test et modification des nom des méthodes de tests. Modification de la section test du rapport</t>
+  </si>
+  <si>
+    <t>Modification de certains commentaires du code</t>
   </si>
 </sst>
 </file>
@@ -1235,7 +1238,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>405</c:v>
+                  <c:v>435</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -2159,16 +2162,16 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>4.6692607003891051E-2</c:v>
+                  <c:v>4.5627376425855515E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.63813229571984431</c:v>
+                  <c:v>0.62357414448669202</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.31517509727626458</c:v>
+                  <c:v>0.33079847908745247</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -4406,7 +4409,7 @@
       <c r="B3" s="86"/>
       <c r="C3" s="67" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>21 heures 55 minutes</v>
+        <v>22 heures 25 minutes</v>
       </c>
       <c r="D3" s="17"/>
       <c r="E3" s="3"/>
@@ -4425,11 +4428,11 @@
       </c>
       <c r="D4" s="17">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>475</v>
+        <v>505</v>
       </c>
       <c r="E4" s="24">
         <f>SUM(C4:D4)</f>
-        <v>1315</v>
+        <v>1345</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -5085,15 +5088,23 @@
       <c r="G32" s="39"/>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A33" s="63" t="str">
+      <c r="A33" s="63">
         <f>IF(ISBLANK(B33),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B33))</f>
-        <v/>
-      </c>
-      <c r="B33" s="34"/>
+        <v>41</v>
+      </c>
+      <c r="B33" s="34">
+        <v>46300</v>
+      </c>
       <c r="C33" s="35"/>
-      <c r="D33" s="36"/>
-      <c r="E33" s="37"/>
-      <c r="F33" s="22"/>
+      <c r="D33" s="36">
+        <v>30</v>
+      </c>
+      <c r="E33" s="37" t="s">
+        <v>17</v>
+      </c>
+      <c r="F33" s="22" t="s">
+        <v>59</v>
+      </c>
       <c r="G33" s="40"/>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
@@ -11238,7 +11249,7 @@
       </c>
       <c r="G6" s="72">
         <f>SUM(A6:B6)/$C$11</f>
-        <v>4.6692607003891051E-2</v>
+        <v>4.5627376425855515E-2</v>
       </c>
       <c r="L6" s="51" t="str">
         <f>'Journal de travail'!M8</f>
@@ -11275,7 +11286,7 @@
       </c>
       <c r="G7" s="75">
         <f t="shared" ref="G7:G9" si="2">SUM(A7:B7)/$C$11</f>
-        <v>0.63813229571984431</v>
+        <v>0.62357414448669202</v>
       </c>
       <c r="L7" s="53" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11333,11 +11344,11 @@
       </c>
       <c r="B9">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E9,'Journal de travail'!$D$7:$D$532)</f>
-        <v>105</v>
+        <v>135</v>
       </c>
       <c r="C9">
         <f t="shared" si="0"/>
-        <v>405</v>
+        <v>435</v>
       </c>
       <c r="E9" s="77" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11345,11 +11356,11 @@
       </c>
       <c r="F9" s="74" t="str">
         <f t="shared" si="1"/>
-        <v>6 h 45 min</v>
+        <v>7 h 15 min</v>
       </c>
       <c r="G9" s="75">
         <f t="shared" si="2"/>
-        <v>0.31517509727626458</v>
+        <v>0.33079847908745247</v>
       </c>
       <c r="L9" s="55" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11405,22 +11416,22 @@
       </c>
       <c r="B11">
         <f>SUM(B6:B10)</f>
-        <v>445</v>
+        <v>475</v>
       </c>
       <c r="C11">
         <f>SUM(A11:B11)</f>
-        <v>1285</v>
+        <v>1315</v>
       </c>
       <c r="E11" s="81" t="s">
         <v>29</v>
       </c>
       <c r="F11" s="71" t="str">
         <f t="shared" si="1"/>
-        <v>21 h 25 min</v>
+        <v>21 h 55 min</v>
       </c>
       <c r="G11" s="82">
         <f>C11/C12</f>
-        <v>0.24337121212121213</v>
+        <v>0.2490530303030303</v>
       </c>
       <c r="L11" s="56" t="s">
         <v>29</v>
@@ -11459,12 +11470,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="4356f79f-5386-4bda-9d92-82d8bd7b074e" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3eb094ff-ec8d-44d8-be06-94ad3ec8832a">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -11669,20 +11682,21 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="4356f79f-5386-4bda-9d92-82d8bd7b074e" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3eb094ff-ec8d-44d8-be06-94ad3ec8832a">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="4356f79f-5386-4bda-9d92-82d8bd7b074e"/>
+    <ds:schemaRef ds:uri="3eb094ff-ec8d-44d8-be06-94ad3ec8832a"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -11707,12 +11721,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="4356f79f-5386-4bda-9d92-82d8bd7b074e"/>
-    <ds:schemaRef ds:uri="3eb094ff-ec8d-44d8-be06-94ad3ec8832a"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
refactor(ShowTable) : Modidication de l'affichage du tableau pour que ce sois responsive selon la taille du parking
</commit_message>
<xml_diff>
--- a/fichiers/P_parking-jdt-HugoSchweizer.xlsx
+++ b/fichiers/P_parking-jdt-HugoSchweizer.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\P_parking\fichiers\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\P_parking\fichiers\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B75835B-DC62-4A41-A425-82978D5DC5F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A92B6459-CA98-4E84-A1D0-F6EBE02AEDEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal de travail" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="61">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -222,6 +222,9 @@
   </si>
   <si>
     <t>Modification de certains commentaires du code</t>
+  </si>
+  <si>
+    <t>Modification du fonctionnement de ma méthode qui affiche le tableau</t>
   </si>
 </sst>
 </file>
@@ -984,7 +987,7 @@
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="fr-FR"/>
+  <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -1232,7 +1235,7 @@
                   <c:v>60</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>820</c:v>
+                  <c:v>850</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -1350,7 +1353,7 @@
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="fr-FR"/>
+  <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -1723,7 +1726,7 @@
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="fr-FR"/>
+  <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -2162,16 +2165,16 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>4.5627376425855515E-2</c:v>
+                  <c:v>4.4609665427509292E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.62357414448669202</c:v>
+                  <c:v>0.63197026022304836</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.33079847908745247</c:v>
+                  <c:v>0.32342007434944237</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -4357,7 +4360,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8FF2E8F1-C793-7E43-B3DE-C075053A97DA}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:O532"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.5" style="7" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11.875" style="1" customWidth="1"/>
@@ -4409,7 +4412,7 @@
       <c r="B3" s="86"/>
       <c r="C3" s="67" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>22 heures 25 minutes</v>
+        <v>22 heures 55 minutes</v>
       </c>
       <c r="D3" s="17"/>
       <c r="E3" s="3"/>
@@ -4428,11 +4431,11 @@
       </c>
       <c r="D4" s="17">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>505</v>
+        <v>535</v>
       </c>
       <c r="E4" s="24">
         <f>SUM(C4:D4)</f>
-        <v>1345</v>
+        <v>1375</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -5108,16 +5111,26 @@
       <c r="G33" s="40"/>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A34" s="62" t="str">
+      <c r="A34" s="62">
         <f>IF(ISBLANK(B34),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B34))</f>
-        <v/>
-      </c>
-      <c r="B34" s="30"/>
+        <v>41</v>
+      </c>
+      <c r="B34" s="30">
+        <v>46300</v>
+      </c>
       <c r="C34" s="31"/>
-      <c r="D34" s="32"/>
-      <c r="E34" s="33"/>
-      <c r="F34" s="22"/>
-      <c r="G34" s="39"/>
+      <c r="D34" s="32">
+        <v>30</v>
+      </c>
+      <c r="E34" s="33" t="s">
+        <v>16</v>
+      </c>
+      <c r="F34" s="22" t="s">
+        <v>60</v>
+      </c>
+      <c r="G34" s="39" t="s">
+        <v>53</v>
+      </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="63" t="str">
@@ -11155,7 +11168,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D21D7432-C939-0D45-BAC2-A6A2196EA9C6}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A2:N13"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="3" width="10.875" hidden="1" customWidth="1"/>
     <col min="4" max="4" width="10.875" customWidth="1"/>
@@ -11249,7 +11262,7 @@
       </c>
       <c r="G6" s="72">
         <f>SUM(A6:B6)/$C$11</f>
-        <v>4.5627376425855515E-2</v>
+        <v>4.4609665427509292E-2</v>
       </c>
       <c r="L6" s="51" t="str">
         <f>'Journal de travail'!M8</f>
@@ -11270,11 +11283,11 @@
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$D$7:$D$532)</f>
-        <v>340</v>
+        <v>370</v>
       </c>
       <c r="C7">
         <f t="shared" si="0"/>
-        <v>820</v>
+        <v>850</v>
       </c>
       <c r="E7" s="73" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11282,11 +11295,11 @@
       </c>
       <c r="F7" s="74" t="str">
         <f t="shared" ref="F7:F11" si="1">QUOTIENT(SUM(A7:B7),60)&amp;" h "&amp;TEXT(MOD(SUM(A7:B7),60), "00")&amp;" min"</f>
-        <v>13 h 40 min</v>
+        <v>14 h 10 min</v>
       </c>
       <c r="G7" s="75">
         <f t="shared" ref="G7:G9" si="2">SUM(A7:B7)/$C$11</f>
-        <v>0.62357414448669202</v>
+        <v>0.63197026022304836</v>
       </c>
       <c r="L7" s="53" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11360,7 +11373,7 @@
       </c>
       <c r="G9" s="75">
         <f t="shared" si="2"/>
-        <v>0.33079847908745247</v>
+        <v>0.32342007434944237</v>
       </c>
       <c r="L9" s="55" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11416,22 +11429,22 @@
       </c>
       <c r="B11">
         <f>SUM(B6:B10)</f>
-        <v>475</v>
+        <v>505</v>
       </c>
       <c r="C11">
         <f>SUM(A11:B11)</f>
-        <v>1315</v>
+        <v>1345</v>
       </c>
       <c r="E11" s="81" t="s">
         <v>29</v>
       </c>
       <c r="F11" s="71" t="str">
         <f t="shared" si="1"/>
-        <v>21 h 55 min</v>
+        <v>22 h 25 min</v>
       </c>
       <c r="G11" s="82">
         <f>C11/C12</f>
-        <v>0.2490530303030303</v>
+        <v>0.25473484848484851</v>
       </c>
       <c r="L11" s="56" t="s">
         <v>29</v>
@@ -11461,7 +11474,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67F31118-7D2C-C547-B9C9-EA2B04E048B8}">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <sheetProtection algorithmName="SHA-512" hashValue="hkKOZ8xr/Okjo/AJlNTtoGYYhES8sIn2fOpGKGGyPJqhNRzaMuj9V6Pke+VqLSypQTwaNPCt0dhRPEVp9CfBFA==" saltValue="lF/ApQWS3LBdJp0wgcNUcQ==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -11470,14 +11483,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="4356f79f-5386-4bda-9d92-82d8bd7b074e" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3eb094ff-ec8d-44d8-be06-94ad3ec8832a">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -11682,21 +11693,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="4356f79f-5386-4bda-9d92-82d8bd7b074e" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3eb094ff-ec8d-44d8-be06-94ad3ec8832a">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="4356f79f-5386-4bda-9d92-82d8bd7b074e"/>
-    <ds:schemaRef ds:uri="3eb094ff-ec8d-44d8-be06-94ad3ec8832a"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -11721,9 +11731,12 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="4356f79f-5386-4bda-9d92-82d8bd7b074e"/>
+    <ds:schemaRef ds:uri="3eb094ff-ec8d-44d8-be06-94ad3ec8832a"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
refactor(ShowTable) : Modification du fonctionnement de ma méthode qui affiche le tableau pour qu'il soie responsive selon la taille du tableau
</commit_message>
<xml_diff>
--- a/fichiers/P_parking-jdt-HugoSchweizer.xlsx
+++ b/fichiers/P_parking-jdt-HugoSchweizer.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\P_parking\fichiers\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A92B6459-CA98-4E84-A1D0-F6EBE02AEDEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7542514-659C-40F9-B6D9-2AACFED540F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="62">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -225,6 +225,9 @@
   </si>
   <si>
     <t>Modification du fonctionnement de ma méthode qui affiche le tableau</t>
+  </si>
+  <si>
+    <t>Modification du fonctionnement de ma méthode qui affiche le tableau pour qu'il soie responsive selon la taille du tableau</t>
   </si>
 </sst>
 </file>
@@ -1235,7 +1238,7 @@
                   <c:v>60</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>850</c:v>
+                  <c:v>865</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -2165,16 +2168,16 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>4.4609665427509292E-2</c:v>
+                  <c:v>4.4117647058823532E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.63197026022304836</c:v>
+                  <c:v>0.63602941176470584</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.32342007434944237</c:v>
+                  <c:v>0.31985294117647056</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -4412,7 +4415,7 @@
       <c r="B3" s="86"/>
       <c r="C3" s="67" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>22 heures 55 minutes</v>
+        <v>23 heures 10 minutes</v>
       </c>
       <c r="D3" s="17"/>
       <c r="E3" s="3"/>
@@ -4431,11 +4434,11 @@
       </c>
       <c r="D4" s="17">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>535</v>
+        <v>550</v>
       </c>
       <c r="E4" s="24">
         <f>SUM(C4:D4)</f>
-        <v>1375</v>
+        <v>1390</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -5132,17 +5135,27 @@
         <v>53</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A35" s="63" t="str">
+    <row r="35" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A35" s="63">
         <f>IF(ISBLANK(B35),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B35))</f>
-        <v/>
-      </c>
-      <c r="B35" s="34"/>
+        <v>41</v>
+      </c>
+      <c r="B35" s="34">
+        <v>46302</v>
+      </c>
       <c r="C35" s="35"/>
-      <c r="D35" s="36"/>
-      <c r="E35" s="37"/>
-      <c r="F35" s="23"/>
-      <c r="G35" s="40"/>
+      <c r="D35" s="36">
+        <v>15</v>
+      </c>
+      <c r="E35" s="37" t="s">
+        <v>16</v>
+      </c>
+      <c r="F35" s="23" t="s">
+        <v>61</v>
+      </c>
+      <c r="G35" s="40" t="s">
+        <v>53</v>
+      </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="62" t="str">
@@ -11262,7 +11275,7 @@
       </c>
       <c r="G6" s="72">
         <f>SUM(A6:B6)/$C$11</f>
-        <v>4.4609665427509292E-2</v>
+        <v>4.4117647058823532E-2</v>
       </c>
       <c r="L6" s="51" t="str">
         <f>'Journal de travail'!M8</f>
@@ -11283,11 +11296,11 @@
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$D$7:$D$532)</f>
-        <v>370</v>
+        <v>385</v>
       </c>
       <c r="C7">
         <f t="shared" si="0"/>
-        <v>850</v>
+        <v>865</v>
       </c>
       <c r="E7" s="73" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11295,11 +11308,11 @@
       </c>
       <c r="F7" s="74" t="str">
         <f t="shared" ref="F7:F11" si="1">QUOTIENT(SUM(A7:B7),60)&amp;" h "&amp;TEXT(MOD(SUM(A7:B7),60), "00")&amp;" min"</f>
-        <v>14 h 10 min</v>
+        <v>14 h 25 min</v>
       </c>
       <c r="G7" s="75">
         <f t="shared" ref="G7:G9" si="2">SUM(A7:B7)/$C$11</f>
-        <v>0.63197026022304836</v>
+        <v>0.63602941176470584</v>
       </c>
       <c r="L7" s="53" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11373,7 +11386,7 @@
       </c>
       <c r="G9" s="75">
         <f t="shared" si="2"/>
-        <v>0.32342007434944237</v>
+        <v>0.31985294117647056</v>
       </c>
       <c r="L9" s="55" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11429,22 +11442,22 @@
       </c>
       <c r="B11">
         <f>SUM(B6:B10)</f>
-        <v>505</v>
+        <v>520</v>
       </c>
       <c r="C11">
         <f>SUM(A11:B11)</f>
-        <v>1345</v>
+        <v>1360</v>
       </c>
       <c r="E11" s="81" t="s">
         <v>29</v>
       </c>
       <c r="F11" s="71" t="str">
         <f t="shared" si="1"/>
-        <v>22 h 25 min</v>
+        <v>22 h 40 min</v>
       </c>
       <c r="G11" s="82">
         <f>C11/C12</f>
-        <v>0.25473484848484851</v>
+        <v>0.25757575757575757</v>
       </c>
       <c r="L11" s="56" t="s">
         <v>29</v>
@@ -11483,12 +11496,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="4356f79f-5386-4bda-9d92-82d8bd7b074e" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3eb094ff-ec8d-44d8-be06-94ad3ec8832a">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -11693,20 +11708,21 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="4356f79f-5386-4bda-9d92-82d8bd7b074e" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3eb094ff-ec8d-44d8-be06-94ad3ec8832a">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="4356f79f-5386-4bda-9d92-82d8bd7b074e"/>
+    <ds:schemaRef ds:uri="3eb094ff-ec8d-44d8-be06-94ad3ec8832a"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -11731,12 +11747,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="4356f79f-5386-4bda-9d92-82d8bd7b074e"/>
-    <ds:schemaRef ds:uri="3eb094ff-ec8d-44d8-be06-94ad3ec8832a"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Refactor(EnterVehicule) : Ajouts de texte explicatif pendant l'ajout d'une voiture car les actions q'on devait faire étaient floue. J'ai aussi fait en sorte qu'à chaque fois qu'on affiche la plaque de la voiture, elle s'affiche en majuscule.
</commit_message>
<xml_diff>
--- a/fichiers/P_parking-jdt-HugoSchweizer.xlsx
+++ b/fichiers/P_parking-jdt-HugoSchweizer.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\P_parking\fichiers\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\P_parking\fichiers\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7542514-659C-40F9-B6D9-2AACFED540F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66E66CBD-66F3-479C-805D-34B26F66EB03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal de travail" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="64">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -228,6 +228,13 @@
   </si>
   <si>
     <t>Modification du fonctionnement de ma méthode qui affiche le tableau pour qu'il soie responsive selon la taille du tableau</t>
+  </si>
+  <si>
+    <t>je ne peux pas mettre cette description à la ligne donc je l'ai sautée</t>
+  </si>
+  <si>
+    <t>Ajouts de texte explicatif pendant l'ajout d'une voiture car les actions q'on devait faire étaient floue. 
+J'ai aussi fait en sorte qu'à chaque fois qu'on affiche la plaque de la voiture, elle s'affiche en majuscule.</t>
   </si>
 </sst>
 </file>
@@ -495,7 +502,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="87">
+  <cellXfs count="92">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -692,6 +699,23 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
+      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -990,7 +1014,7 @@
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
+  <c:lang val="fr-FR"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -1238,7 +1262,7 @@
                   <c:v>60</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>865</c:v>
+                  <c:v>880</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -1356,7 +1380,7 @@
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
+  <c:lang val="fr-FR"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -1729,7 +1753,7 @@
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
+  <c:lang val="fr-FR"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -2168,16 +2192,16 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>4.4117647058823532E-2</c:v>
+                  <c:v>4.363636363636364E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.63602941176470584</c:v>
+                  <c:v>0.64</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.31985294117647056</c:v>
+                  <c:v>0.31636363636363635</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -4363,7 +4387,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8FF2E8F1-C793-7E43-B3DE-C075053A97DA}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:O532"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.5" style="7" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11.875" style="1" customWidth="1"/>
@@ -4415,7 +4439,7 @@
       <c r="B3" s="86"/>
       <c r="C3" s="67" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>23 heures 10 minutes</v>
+        <v>23 heures 25 minutes</v>
       </c>
       <c r="D3" s="17"/>
       <c r="E3" s="3"/>
@@ -4434,11 +4458,11 @@
       </c>
       <c r="D4" s="17">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>550</v>
+        <v>565</v>
       </c>
       <c r="E4" s="24">
         <f>SUM(C4:D4)</f>
-        <v>1390</v>
+        <v>1405</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -5027,7 +5051,9 @@
       <c r="D29" s="36"/>
       <c r="E29" s="37"/>
       <c r="F29" s="22"/>
-      <c r="G29" s="40"/>
+      <c r="G29" s="40" t="s">
+        <v>62</v>
+      </c>
     </row>
     <row r="30" spans="1:15" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A30" s="62">
@@ -5157,28 +5183,36 @@
         <v>53</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A36" s="62" t="str">
-        <f>IF(ISBLANK(B36),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B36))</f>
-        <v/>
-      </c>
-      <c r="B36" s="30"/>
-      <c r="C36" s="31"/>
-      <c r="D36" s="32"/>
-      <c r="E36" s="33"/>
-      <c r="F36" s="22"/>
+    <row r="36" spans="1:7" ht="63" x14ac:dyDescent="0.25">
+      <c r="A36" s="62">
+        <f>IF(ISBLANK(B37),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B37))</f>
+        <v>41</v>
+      </c>
+      <c r="B36" s="87"/>
+      <c r="C36" s="88"/>
+      <c r="D36" s="32">
+        <v>15</v>
+      </c>
+      <c r="E36" s="33" t="s">
+        <v>16</v>
+      </c>
+      <c r="F36" s="23" t="s">
+        <v>63</v>
+      </c>
       <c r="G36" s="39"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A37" s="63" t="str">
-        <f>IF(ISBLANK(B37),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B37))</f>
-        <v/>
-      </c>
-      <c r="B37" s="34"/>
-      <c r="C37" s="35"/>
-      <c r="D37" s="36"/>
-      <c r="E37" s="37"/>
-      <c r="F37" s="22"/>
+      <c r="A37" s="63" t="e">
+        <f>IF(ISBLANK(#REF!),"",_xlfn.ISOWEEKNUM('Journal de travail'!#REF!))</f>
+        <v>#REF!</v>
+      </c>
+      <c r="B37" s="30">
+        <v>46304</v>
+      </c>
+      <c r="C37" s="31"/>
+      <c r="D37" s="89"/>
+      <c r="E37" s="90"/>
+      <c r="F37" s="91"/>
       <c r="G37" s="40"/>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
@@ -5188,9 +5222,9 @@
       </c>
       <c r="B38" s="30"/>
       <c r="C38" s="31"/>
-      <c r="D38" s="32"/>
-      <c r="E38" s="33"/>
-      <c r="F38" s="22"/>
+      <c r="D38" s="89"/>
+      <c r="E38" s="90"/>
+      <c r="F38" s="91"/>
       <c r="G38" s="39"/>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
@@ -11129,7 +11163,7 @@
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="A3:B3"/>
   </mergeCells>
-  <conditionalFormatting sqref="E7:E532">
+  <conditionalFormatting sqref="E39:E532 E7:E36">
     <cfRule type="expression" dxfId="8" priority="1">
       <formula>$E7="Absent"</formula>
     </cfRule>
@@ -11159,13 +11193,13 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C7:C532" xr:uid="{9D52E29F-610D-40B2-B3CC-F94A741DD978}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C7:C35 C37:C532" xr:uid="{9D52E29F-610D-40B2-B3CC-F94A741DD978}">
       <formula1>$N$7:$N$15</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D7:D532" xr:uid="{46510F84-8BCC-4BD6-9A19-9F03ACD74D05}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D7:D36 D39:D532" xr:uid="{46510F84-8BCC-4BD6-9A19-9F03ACD74D05}">
       <formula1>$O$7:$O$19</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E7:E532" xr:uid="{EBCA439E-C5F1-BC4C-88EE-2BB045537E3E}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E7:E36 E39:E532" xr:uid="{EBCA439E-C5F1-BC4C-88EE-2BB045537E3E}">
       <formula1>$M$7:$M$12</formula1>
     </dataValidation>
   </dataValidations>
@@ -11181,7 +11215,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D21D7432-C939-0D45-BAC2-A6A2196EA9C6}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A2:N13"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="3" width="10.875" hidden="1" customWidth="1"/>
     <col min="4" max="4" width="10.875" customWidth="1"/>
@@ -11275,7 +11309,7 @@
       </c>
       <c r="G6" s="72">
         <f>SUM(A6:B6)/$C$11</f>
-        <v>4.4117647058823532E-2</v>
+        <v>4.363636363636364E-2</v>
       </c>
       <c r="L6" s="51" t="str">
         <f>'Journal de travail'!M8</f>
@@ -11296,11 +11330,11 @@
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$D$7:$D$532)</f>
-        <v>385</v>
+        <v>400</v>
       </c>
       <c r="C7">
         <f t="shared" si="0"/>
-        <v>865</v>
+        <v>880</v>
       </c>
       <c r="E7" s="73" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11308,11 +11342,11 @@
       </c>
       <c r="F7" s="74" t="str">
         <f t="shared" ref="F7:F11" si="1">QUOTIENT(SUM(A7:B7),60)&amp;" h "&amp;TEXT(MOD(SUM(A7:B7),60), "00")&amp;" min"</f>
-        <v>14 h 25 min</v>
+        <v>14 h 40 min</v>
       </c>
       <c r="G7" s="75">
         <f t="shared" ref="G7:G9" si="2">SUM(A7:B7)/$C$11</f>
-        <v>0.63602941176470584</v>
+        <v>0.64</v>
       </c>
       <c r="L7" s="53" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11386,7 +11420,7 @@
       </c>
       <c r="G9" s="75">
         <f t="shared" si="2"/>
-        <v>0.31985294117647056</v>
+        <v>0.31636363636363635</v>
       </c>
       <c r="L9" s="55" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11442,22 +11476,22 @@
       </c>
       <c r="B11">
         <f>SUM(B6:B10)</f>
-        <v>520</v>
+        <v>535</v>
       </c>
       <c r="C11">
         <f>SUM(A11:B11)</f>
-        <v>1360</v>
+        <v>1375</v>
       </c>
       <c r="E11" s="81" t="s">
         <v>29</v>
       </c>
       <c r="F11" s="71" t="str">
         <f t="shared" si="1"/>
-        <v>22 h 40 min</v>
+        <v>22 h 55 min</v>
       </c>
       <c r="G11" s="82">
         <f>C11/C12</f>
-        <v>0.25757575757575757</v>
+        <v>0.26041666666666669</v>
       </c>
       <c r="L11" s="56" t="s">
         <v>29</v>
@@ -11487,7 +11521,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67F31118-7D2C-C547-B9C9-EA2B04E048B8}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <sheetProtection algorithmName="SHA-512" hashValue="hkKOZ8xr/Okjo/AJlNTtoGYYhES8sIn2fOpGKGGyPJqhNRzaMuj9V6Pke+VqLSypQTwaNPCt0dhRPEVp9CfBFA==" saltValue="lF/ApQWS3LBdJp0wgcNUcQ==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -11496,14 +11530,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="4356f79f-5386-4bda-9d92-82d8bd7b074e" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3eb094ff-ec8d-44d8-be06-94ad3ec8832a">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -11708,21 +11740,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="4356f79f-5386-4bda-9d92-82d8bd7b074e" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3eb094ff-ec8d-44d8-be06-94ad3ec8832a">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="4356f79f-5386-4bda-9d92-82d8bd7b074e"/>
-    <ds:schemaRef ds:uri="3eb094ff-ec8d-44d8-be06-94ad3ec8832a"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -11747,9 +11778,12 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="4356f79f-5386-4bda-9d92-82d8bd7b074e"/>
+    <ds:schemaRef ds:uri="3eb094ff-ec8d-44d8-be06-94ad3ec8832a"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>